<commit_message>
Update data-ta.xlsx task successes
</commit_message>
<xml_diff>
--- a/g1-09-ta/data-ta.xlsx
+++ b/g1-09-ta/data-ta.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sven\Documents\School\Radboud\Computing Science\Minor\Vakken\Human-Computer Interaction\Ex3\hci-ex3\g1-09-ta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1B07500-48D8-4F73-84F3-6BE8AFEF0AE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDF4199A-FAAD-4B86-BF43-79834F93EB31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="503" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="503" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Background Q" sheetId="3" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="170">
   <si>
     <t>Browser</t>
   </si>
@@ -49,12 +49,6 @@
     <t>Percent</t>
   </si>
   <si>
-    <t>3 Register</t>
-  </si>
-  <si>
-    <t>5 Search</t>
-  </si>
-  <si>
     <t>Task Success (Effectiveness: 0=failure, 1=success)</t>
   </si>
   <si>
@@ -88,9 +82,6 @@
     <t>Median</t>
   </si>
   <si>
-    <t>4 Log In</t>
-  </si>
-  <si>
     <t>Student</t>
   </si>
   <si>
@@ -115,9 +106,6 @@
     <t>1 First Impressions</t>
   </si>
   <si>
-    <t>2 Contact Person</t>
-  </si>
-  <si>
     <t>2 Quality</t>
   </si>
   <si>
@@ -410,21 +398,6 @@
   </si>
   <si>
     <t>woman</t>
-  </si>
-  <si>
-    <t>“Stuart”</t>
-  </si>
-  <si>
-    <t>“Silvia”</t>
-  </si>
-  <si>
-    <t>“Sally”</t>
-  </si>
-  <si>
-    <t>“Martin”</t>
-  </si>
-  <si>
-    <t>“John”</t>
   </si>
   <si>
     <t>Home → Shipping → Delivery</t>
@@ -567,6 +540,18 @@
   </si>
   <si>
     <t>N/A</t>
+  </si>
+  <si>
+    <t>2 Find product</t>
+  </si>
+  <si>
+    <t>3 Best of one</t>
+  </si>
+  <si>
+    <t>4 Build PC</t>
+  </si>
+  <si>
+    <t>5 Account</t>
   </si>
 </sst>
 </file>
@@ -1533,156 +1518,156 @@
   <sheetData>
     <row r="1" spans="1:26" ht="13" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:26" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="C3" s="9" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D3" s="10"/>
       <c r="E3" s="10"/>
       <c r="F3" s="9" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G3" s="11"/>
       <c r="H3" s="9" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="I3" s="10"/>
       <c r="J3" s="10"/>
       <c r="K3" s="9" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="L3" s="10"/>
       <c r="M3" s="10"/>
       <c r="N3" s="9" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="O3" s="10"/>
       <c r="P3" s="10"/>
       <c r="Q3" s="9" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="R3" s="10"/>
       <c r="S3" s="10"/>
       <c r="T3" s="10"/>
       <c r="U3" s="76" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="V3" s="77"/>
       <c r="W3" s="78"/>
       <c r="X3" s="76" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="Y3" s="78"/>
       <c r="Z3" s="11"/>
     </row>
     <row r="4" spans="1:26" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="31" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="D4" s="72" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="D4" s="72" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4" s="12" t="s">
+      <c r="F4" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="H4" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="7" t="s">
-        <v>117</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="H4" s="12" t="s">
+      <c r="I4" s="71" t="s">
+        <v>92</v>
+      </c>
+      <c r="J4" s="72" t="s">
+        <v>93</v>
+      </c>
+      <c r="K4" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="L4" s="71" t="s">
+        <v>92</v>
+      </c>
+      <c r="M4" s="72" t="s">
+        <v>93</v>
+      </c>
+      <c r="N4" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="O4" s="71" t="s">
+        <v>92</v>
+      </c>
+      <c r="P4" s="72" t="s">
+        <v>93</v>
+      </c>
+      <c r="Q4" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="R4" s="13" t="s">
         <v>12</v>
-      </c>
-      <c r="I4" s="71" t="s">
-        <v>96</v>
-      </c>
-      <c r="J4" s="72" t="s">
-        <v>97</v>
-      </c>
-      <c r="K4" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="L4" s="71" t="s">
-        <v>96</v>
-      </c>
-      <c r="M4" s="72" t="s">
-        <v>97</v>
-      </c>
-      <c r="N4" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="O4" s="71" t="s">
-        <v>96</v>
-      </c>
-      <c r="P4" s="72" t="s">
-        <v>97</v>
-      </c>
-      <c r="Q4" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="R4" s="13" t="s">
-        <v>14</v>
       </c>
       <c r="S4" s="13" t="s">
         <v>0</v>
       </c>
       <c r="T4" s="75" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="U4" s="13" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="V4" s="13" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="W4" s="13" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="X4" s="13" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="Y4" s="13" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="Z4" s="14" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B5" s="38" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="C5" s="73" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="D5" s="52">
         <v>19</v>
       </c>
       <c r="E5" s="38" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="H5" s="41" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="I5" s="52">
         <v>5</v>
@@ -1691,7 +1676,7 @@
         <v>7</v>
       </c>
       <c r="K5" s="41" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="L5" s="52">
         <v>15</v>
@@ -1700,7 +1685,7 @@
         <v>28</v>
       </c>
       <c r="N5" s="41" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="O5" s="52">
         <v>10</v>
@@ -1709,60 +1694,60 @@
         <v>28</v>
       </c>
       <c r="Q5" s="42" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="R5" s="16" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="S5" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="T5" s="16">
         <v>4</v>
       </c>
       <c r="U5" s="43" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="V5" s="43" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="W5" s="43" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="X5" s="43" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="Y5" s="43" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="Z5" s="43" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B6" s="38" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="C6" s="73" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="D6" s="52">
         <v>24</v>
       </c>
       <c r="E6" s="38" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
       <c r="H6" s="41" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="I6" s="52">
         <v>10</v>
@@ -1771,7 +1756,7 @@
         <v>35</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="L6" s="52">
         <v>15</v>
@@ -1780,7 +1765,7 @@
         <v>25</v>
       </c>
       <c r="N6" s="15" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="O6" s="52">
         <v>12</v>
@@ -1789,69 +1774,69 @@
         <v>25</v>
       </c>
       <c r="Q6" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="R6" s="4" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="S6" s="4" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="T6" s="4">
         <v>15</v>
       </c>
       <c r="U6" s="43" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="V6" s="4" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="W6" s="4" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="X6" s="43" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="Y6" s="4" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="Z6" s="43" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B7" s="38" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="C7" s="73" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="D7" s="52">
         <v>19</v>
       </c>
       <c r="E7" s="38" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="I7" s="52">
         <v>8</v>
       </c>
       <c r="J7" s="52" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="K7" s="15" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="L7" s="52">
         <v>30</v>
@@ -1860,7 +1845,7 @@
         <v>60</v>
       </c>
       <c r="N7" s="15" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="O7" s="52">
         <v>12</v>
@@ -1869,60 +1854,60 @@
         <v>60</v>
       </c>
       <c r="Q7" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="R7" s="4" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="S7" s="4" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="T7" s="4">
         <v>20</v>
       </c>
       <c r="U7" s="43" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="V7" s="4" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="W7" s="4" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="X7" s="43" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="Y7" s="4" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="Z7" s="43" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B8" s="38" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="C8" s="73" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="D8" s="52">
         <v>29</v>
       </c>
       <c r="E8" s="38" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="H8" s="15" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="I8" s="52">
         <v>15</v>
@@ -1931,7 +1916,7 @@
         <v>55</v>
       </c>
       <c r="K8" s="15" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="L8" s="52">
         <v>0</v>
@@ -1940,7 +1925,7 @@
         <v>21</v>
       </c>
       <c r="N8" s="15" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="O8" s="52">
         <v>14</v>
@@ -1949,10 +1934,10 @@
         <v>21</v>
       </c>
       <c r="Q8" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="R8" s="4" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="S8" s="4" t="s">
         <v>1</v>
@@ -1961,48 +1946,48 @@
         <v>30</v>
       </c>
       <c r="U8" s="43" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="V8" s="4" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="W8" s="4" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="X8" s="43" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="Y8" s="4" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="Z8" s="43" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B9" s="62" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="C9" s="74" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="D9" s="53">
         <v>24</v>
       </c>
       <c r="E9" s="38" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F9" s="20" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="G9" s="20" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="H9" s="21" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="I9" s="54">
         <v>15</v>
@@ -2011,7 +1996,7 @@
         <v>56</v>
       </c>
       <c r="K9" s="21" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="L9" s="54">
         <v>0</v>
@@ -2020,7 +2005,7 @@
         <v>14</v>
       </c>
       <c r="N9" s="21" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="O9" s="54">
         <v>12</v>
@@ -2029,34 +2014,34 @@
         <v>14</v>
       </c>
       <c r="Q9" s="22" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="R9" s="20" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="S9" s="22" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="T9" s="20">
         <v>28</v>
       </c>
       <c r="U9" s="20" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="V9" s="20" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="W9" s="20" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="X9" s="61" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="Y9" s="20" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="Z9" s="43" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
@@ -2070,7 +2055,7 @@
     <row r="11" spans="1:26" ht="13" x14ac:dyDescent="0.3">
       <c r="A11" s="24"/>
       <c r="B11" s="26" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C11" s="5"/>
       <c r="D11" s="51">
@@ -2081,7 +2066,7 @@
       <c r="F11" s="17"/>
       <c r="G11" s="17"/>
       <c r="H11" s="40" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="I11" s="45">
         <f>AVERAGE(I5:I9)</f>
@@ -2092,7 +2077,7 @@
         <v>38.25</v>
       </c>
       <c r="K11" s="40" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="L11" s="45">
         <f>AVERAGE(L5:L9)</f>
@@ -2103,7 +2088,7 @@
         <v>29.6</v>
       </c>
       <c r="N11" s="40" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="O11" s="45">
         <f>AVERAGE(O5:O9)</f>
@@ -2116,7 +2101,7 @@
       <c r="Q11" s="17"/>
       <c r="R11" s="17"/>
       <c r="S11" s="40" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="T11" s="45">
         <f>AVERAGE(T5:T9)</f>
@@ -2126,7 +2111,7 @@
     <row r="12" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="24"/>
       <c r="B12" s="26" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C12" s="5"/>
       <c r="D12" s="28">
@@ -2134,7 +2119,7 @@
         <v>24</v>
       </c>
       <c r="H12" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="I12" s="28">
         <f>MEDIAN(I5:I9)</f>
@@ -2145,7 +2130,7 @@
         <v>45</v>
       </c>
       <c r="K12" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="L12" s="28">
         <f>MEDIAN(L5:L9)</f>
@@ -2156,7 +2141,7 @@
         <v>25</v>
       </c>
       <c r="N12" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="O12" s="28">
         <f>MEDIAN(O5:O9)</f>
@@ -2167,7 +2152,7 @@
         <v>25</v>
       </c>
       <c r="S12" s="40" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="T12" s="28">
         <f>MEDIAN(T5:T9)</f>
@@ -2176,13 +2161,13 @@
     </row>
     <row r="13" spans="1:26" x14ac:dyDescent="0.25">
       <c r="H13" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="K13" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="S13" s="40" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="T13" s="40"/>
     </row>
@@ -2213,12 +2198,12 @@
   <sheetData>
     <row r="1" spans="1:7" ht="13" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="13" x14ac:dyDescent="0.3">
       <c r="C3" s="35" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D3" s="36"/>
       <c r="E3" s="37"/>
@@ -2227,33 +2212,33 @@
     </row>
     <row r="4" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="31" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C4" s="25" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D4" s="25" t="s">
-        <v>26</v>
+        <v>166</v>
       </c>
       <c r="E4" s="25" t="s">
-        <v>4</v>
+        <v>167</v>
       </c>
       <c r="F4" s="25" t="s">
-        <v>17</v>
+        <v>168</v>
       </c>
       <c r="G4" s="25" t="s">
-        <v>5</v>
+        <v>169</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B5" s="38" t="s">
-        <v>125</v>
+        <v>141</v>
       </c>
       <c r="C5" s="27">
         <v>1</v>
@@ -2273,22 +2258,22 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B6" s="38" t="s">
-        <v>126</v>
+        <v>142</v>
       </c>
       <c r="C6" s="27">
         <v>1</v>
       </c>
       <c r="D6" s="27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6" s="27">
         <v>1</v>
       </c>
       <c r="F6" s="27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" s="27">
         <v>1</v>
@@ -2296,22 +2281,22 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B7" s="38" t="s">
-        <v>127</v>
+        <v>143</v>
       </c>
       <c r="C7" s="27">
         <v>1</v>
       </c>
       <c r="D7" s="27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" s="27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" s="27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7" s="27">
         <v>1</v>
@@ -2319,22 +2304,22 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B8" s="38" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
       <c r="C8" s="27">
         <v>1</v>
       </c>
       <c r="D8" s="27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" s="27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" s="27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" s="27">
         <v>1</v>
@@ -2342,10 +2327,10 @@
     </row>
     <row r="9" spans="1:7" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="19" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B9" s="62" t="s">
-        <v>129</v>
+        <v>145</v>
       </c>
       <c r="C9" s="27">
         <v>1</v>
@@ -2357,7 +2342,7 @@
         <v>0</v>
       </c>
       <c r="F9" s="27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" s="27">
         <v>1</v>
@@ -2374,7 +2359,7 @@
       </c>
       <c r="D10" s="44">
         <f>SUM(D5:D9)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E10" s="44">
         <f>SUM(E5:E9)</f>
@@ -2400,7 +2385,7 @@
       </c>
       <c r="D11" s="49">
         <f>SUM(D5:D9)/COUNT(D5:D9)</f>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="E11" s="49">
         <f>SUM(E5:E9)/COUNT(E5:E9)</f>
@@ -2440,47 +2425,47 @@
   <sheetData>
     <row r="1" spans="1:11" ht="13" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="13" x14ac:dyDescent="0.3">
       <c r="G3" s="58" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:11" s="56" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="60" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B4" s="60" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C4" s="60" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D4" s="60" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="E4" s="60" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="F4" s="60" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="G4" s="57" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="H4" s="57" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="I4" s="57" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="J4" s="57" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="K4" s="59" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="25" x14ac:dyDescent="0.25">
@@ -2488,19 +2473,19 @@
         <v>1</v>
       </c>
       <c r="B5" s="64" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="C5" s="69" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="D5" s="69" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="E5" s="69" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="F5" s="69" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="G5" s="66">
         <v>2</v>
@@ -2525,19 +2510,19 @@
         <v>2</v>
       </c>
       <c r="B6" s="64" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C6" s="64" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D6" s="63" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="E6" s="63" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F6" s="69" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="G6" s="66">
         <v>3</v>
@@ -2562,19 +2547,19 @@
         <v>3</v>
       </c>
       <c r="B7" s="64" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C7" s="64" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D7" s="63" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E7" s="63" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F7" s="64" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="G7" s="66">
         <v>4</v>
@@ -2599,19 +2584,19 @@
         <v>4</v>
       </c>
       <c r="B8" s="64" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C8" s="64" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="D8" s="63" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E8" s="69" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="F8" s="70" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="G8" s="66">
         <v>3</v>
@@ -2636,19 +2621,19 @@
         <v>5</v>
       </c>
       <c r="B9" s="64" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C9" s="64" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D9" s="63" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E9" s="63" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F9" s="69" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="G9" s="66">
         <v>3</v>
@@ -2672,19 +2657,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="64" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C10" s="64" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="D10" s="63" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E10" s="63" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="F10" s="69" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="G10" s="66">
         <v>2</v>
@@ -2708,19 +2693,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="64" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C11" s="64" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="D11" s="63" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E11" s="63" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F11" s="64" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G11" s="66">
         <v>2</v>
@@ -2741,22 +2726,22 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="68" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B12" s="69" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C12" s="69" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D12" s="65" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E12" s="65" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F12" s="69" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G12" s="66">
         <v>2</v>
@@ -2777,22 +2762,22 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="68" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B13" s="69" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C13" s="69" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D13" s="65" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E13" s="65" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F13" s="69" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G13" s="66">
         <v>2</v>
@@ -2816,19 +2801,19 @@
         <v>21</v>
       </c>
       <c r="B14" s="64" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C14" s="64" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D14" s="65" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E14" s="65" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="F14" s="70" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="G14" s="66">
         <v>1</v>
@@ -2873,47 +2858,47 @@
   <sheetData>
     <row r="1" spans="1:11" ht="13" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="13" x14ac:dyDescent="0.3">
       <c r="G3" s="58" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:11" s="56" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="60" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B4" s="60" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C4" s="60" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D4" s="60" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="E4" s="60" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="F4" s="60" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="G4" s="57" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="H4" s="57" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="I4" s="57" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="J4" s="57" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="K4" s="59" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="37.5" x14ac:dyDescent="0.25">
@@ -2921,19 +2906,19 @@
         <v>1</v>
       </c>
       <c r="B5" s="64" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C5" s="64" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D5" s="69" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="E5" s="69" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="F5" s="69" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="G5" s="66">
         <v>2</v>
@@ -2958,19 +2943,19 @@
         <v>2</v>
       </c>
       <c r="B6" s="64" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C6" s="64" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="D6" s="64" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E6" s="64" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F6" s="69" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="G6" s="66">
         <v>3</v>
@@ -2995,19 +2980,19 @@
         <v>3</v>
       </c>
       <c r="B7" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C7" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D7" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E7" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F7" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G7" s="66">
         <v>4</v>
@@ -3032,19 +3017,19 @@
         <v>4</v>
       </c>
       <c r="B8" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C8" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D8" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E8" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F8" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G8" s="66">
         <v>3</v>
@@ -3069,19 +3054,19 @@
         <v>5</v>
       </c>
       <c r="B9" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C9" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D9" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E9" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F9" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G9" s="66">
         <v>3</v>
@@ -3105,19 +3090,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C10" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D10" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E10" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F10" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G10" s="66">
         <v>2</v>
@@ -3141,19 +3126,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C11" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D11" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E11" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F11" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G11" s="66">
         <v>2</v>
@@ -3177,19 +3162,19 @@
         <v>8</v>
       </c>
       <c r="B12" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C12" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D12" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E12" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F12" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G12" s="66">
         <v>2</v>
@@ -3213,19 +3198,19 @@
         <v>9</v>
       </c>
       <c r="B13" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C13" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D13" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E13" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F13" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G13" s="66">
         <v>2</v>
@@ -3249,19 +3234,19 @@
         <v>10</v>
       </c>
       <c r="B14" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C14" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D14" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E14" s="64" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F14" s="64" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G14" s="66">
         <v>1</v>
@@ -3325,68 +3310,68 @@
   <sheetData>
     <row r="1" spans="1:17" ht="13" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:17" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="31" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C3" s="29" t="s">
+        <v>79</v>
+      </c>
+      <c r="D3" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" s="30" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="H3" s="30" t="s">
+        <v>27</v>
+      </c>
+      <c r="I3" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" s="30" t="s">
+        <v>29</v>
+      </c>
+      <c r="K3" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="L3" s="30" t="s">
+        <v>80</v>
+      </c>
+      <c r="M3" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="N3" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="O3" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="P3" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="D3" s="30" t="s">
-        <v>27</v>
-      </c>
-      <c r="E3" s="30" t="s">
-        <v>28</v>
-      </c>
-      <c r="F3" s="30" t="s">
-        <v>29</v>
-      </c>
-      <c r="G3" s="30" t="s">
-        <v>30</v>
-      </c>
-      <c r="H3" s="30" t="s">
-        <v>31</v>
-      </c>
-      <c r="I3" s="30" t="s">
-        <v>32</v>
-      </c>
-      <c r="J3" s="30" t="s">
-        <v>33</v>
-      </c>
-      <c r="K3" s="30" t="s">
-        <v>34</v>
-      </c>
-      <c r="L3" s="30" t="s">
-        <v>84</v>
-      </c>
-      <c r="M3" s="30" t="s">
-        <v>85</v>
-      </c>
-      <c r="N3" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="O3" s="13" t="s">
-        <v>121</v>
-      </c>
-      <c r="P3" s="13" t="s">
-        <v>87</v>
-      </c>
       <c r="Q3" s="13" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B4" s="38" t="s">
-        <v>125</v>
+        <v>141</v>
       </c>
       <c r="C4" s="32">
         <v>5</v>
@@ -3436,10 +3421,10 @@
     </row>
     <row r="5" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B5" s="38" t="s">
-        <v>126</v>
+        <v>142</v>
       </c>
       <c r="C5" s="32">
         <v>4</v>
@@ -3489,10 +3474,10 @@
     </row>
     <row r="6" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B6" s="38" t="s">
-        <v>127</v>
+        <v>143</v>
       </c>
       <c r="C6" s="32">
         <v>3</v>
@@ -3542,10 +3527,10 @@
     </row>
     <row r="7" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B7" s="38" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
       <c r="C7" s="32">
         <v>2</v>
@@ -3595,10 +3580,10 @@
     </row>
     <row r="8" spans="1:17" s="18" customFormat="1" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="19" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B8" s="62" t="s">
-        <v>129</v>
+        <v>145</v>
       </c>
       <c r="C8" s="33">
         <v>3</v>
@@ -3662,7 +3647,7 @@
     <row r="10" spans="1:17" s="18" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A10" s="24"/>
       <c r="B10" s="24" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C10" s="50">
         <f>AVERAGE(C4:C8)</f>
@@ -3728,7 +3713,7 @@
     <row r="11" spans="1:17" s="18" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="24"/>
       <c r="B11" s="24" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C11" s="34">
         <f>STDEV(C4:C8)</f>

</xml_diff>

<commit_message>
Added TP1 findings to Excel table
</commit_message>
<xml_diff>
--- a/g1-09-ta/data-ta.xlsx
+++ b/g1-09-ta/data-ta.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sven\Documents\School\Radboud\Computing Science\Minor\Vakken\Human-Computer Interaction\Ex3\hci-ex3\g1-09-ta\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Uni\HCI\hci-ex3\g1-09-ta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDF4199A-FAAD-4B86-BF43-79834F93EB31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2EE88A9-A081-42E5-90C7-7784388F1C5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="503" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="503" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Background Q" sheetId="3" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="147">
   <si>
     <t>Browser</t>
   </si>
@@ -145,84 +145,6 @@
     <t>Timestamp(s)</t>
   </si>
   <si>
-    <t>Stimulus Satiation</t>
-  </si>
-  <si>
-    <t>too much stimuli on the first page</t>
-  </si>
-  <si>
-    <t>Home page</t>
-  </si>
-  <si>
-    <t>Too Much Information For Catalogue Needed</t>
-  </si>
-  <si>
-    <t>you have to enter too much information to order a catalogue</t>
-  </si>
-  <si>
-    <t>Discount</t>
-  </si>
-  <si>
-    <t>just 295,90 instead of 295,95</t>
-  </si>
-  <si>
-    <t>Location Of Stores</t>
-  </si>
-  <si>
-    <t>user didn't see on first sight where all the stores are located</t>
-  </si>
-  <si>
-    <t>Annoying Pop-UP Window</t>
-  </si>
-  <si>
-    <t>annoying pop-up window when you visit the site</t>
-  </si>
-  <si>
-    <t>pops up when you visit web site with an unknown ip adress</t>
-  </si>
-  <si>
-    <t>No Catalogue Name</t>
-  </si>
-  <si>
-    <t>HR</t>
-  </si>
-  <si>
-    <t>CT</t>
-  </si>
-  <si>
-    <t>TG</t>
-  </si>
-  <si>
-    <t>SS</t>
-  </si>
-  <si>
-    <t>Unsure which catalogue, since no name is displayed.</t>
-  </si>
-  <si>
-    <t>TP2 00:06:04</t>
-  </si>
-  <si>
-    <t>TP3 00:09:55</t>
-  </si>
-  <si>
-    <t>TP4 00:13:55, TP5 00:15:10</t>
-  </si>
-  <si>
-    <t>TP3 00:05:48</t>
-  </si>
-  <si>
-    <t>TP2 00:13:51</t>
-  </si>
-  <si>
-    <t>TP5 00:02:56</t>
-  </si>
-  <si>
-    <t>Shipping Link not to Shipping Costs</t>
-  </si>
-  <si>
-    <t>When shipping link was clicked products were shown.</t>
-  </si>
-  <si>
     <t>Location (How Reproducible?)</t>
   </si>
   <si>
@@ -244,33 +166,6 @@
     <t>Positivity</t>
   </si>
   <si>
-    <t>...</t>
-  </si>
-  <si>
-    <t>Clear Registration Page</t>
-  </si>
-  <si>
-    <t>The registration page is well laid out and clear.</t>
-  </si>
-  <si>
-    <t>The contact information is...</t>
-  </si>
-  <si>
-    <t>Good Contact Information</t>
-  </si>
-  <si>
-    <t>TP2 00:12:48</t>
-  </si>
-  <si>
-    <t>p02-tp2-contact.mp4</t>
-  </si>
-  <si>
-    <t>n02-tp2-shipping.mp4</t>
-  </si>
-  <si>
-    <t>n21-tp2-cat-name.mp4</t>
-  </si>
-  <si>
     <t>Mean</t>
   </si>
   <si>
@@ -400,55 +295,6 @@
     <t>woman</t>
   </si>
   <si>
-    <t>Home → Shipping → Delivery</t>
-  </si>
-  <si>
-    <t>Home → Store Finder</t>
-  </si>
-  <si>
-    <t>Any product page, link “Shipping”.</t>
-  </si>
-  <si>
-    <t>product page for “Blue Ski Jacket”</t>
-  </si>
-  <si>
-    <t>https://example.com/en/page.bto?page=catalog</t>
-  </si>
-  <si>
-    <t>Home → Register</t>
-  </si>
-  <si>
-    <t>Home → Contact</t>
-  </si>
-  <si>
-    <t>Unclear When Free Delivery Applies</t>
-  </si>
-  <si>
-    <t>Contradictory information: "free delivery" or "free delivery above €200"</t>
-  </si>
-  <si>
-    <t>p01-tp1-reg-clear.mp4,
-p01-tp3-reg-clear.mp4,
-p01-tp4-reg-clear.mp4</t>
-  </si>
-  <si>
-    <t>TP1 00:01:15,
-TP3 01:24:36,
-TP4 01:26:40</t>
-  </si>
-  <si>
-    <t>n01-tp4-unclear-when-delivery-free.mp4,
-n01-tp5-unclear-when-delivery-free.mp4</t>
-  </si>
-  <si>
-    <t>TP4 00:03:00,
-TP5 00:01:50</t>
-  </si>
-  <si>
-    <t>TP4 00:13:55,
-TP5 00:15:10</t>
-  </si>
-  <si>
     <t>Area of Study</t>
   </si>
   <si>
@@ -552,6 +398,84 @@
   </si>
   <si>
     <t>5 Account</t>
+  </si>
+  <si>
+    <t>The interface element "Spare mit Rabattcodes" remains in German even when the website is set to English</t>
+  </si>
+  <si>
+    <t>Wrong Language Text</t>
+  </si>
+  <si>
+    <t>TP1 00:02:00</t>
+  </si>
+  <si>
+    <t>SJ</t>
+  </si>
+  <si>
+    <t>LR</t>
+  </si>
+  <si>
+    <t>DC</t>
+  </si>
+  <si>
+    <t>FM</t>
+  </si>
+  <si>
+    <t>Homepage → scroll down to category "Spare mit Rabattcodes"</t>
+  </si>
+  <si>
+    <t>When the user searches for a MacBook, they note that the search results appear visually similar at first glance</t>
+  </si>
+  <si>
+    <t>Visually Similar Search Results</t>
+  </si>
+  <si>
+    <t>TP1 00:05:31</t>
+  </si>
+  <si>
+    <t>Search for "apple laptop 128gb ram"</t>
+  </si>
+  <si>
+    <t>Comparison Labels Overlap Content</t>
+  </si>
+  <si>
+    <t>Scrolling horizontally within the comparison element causes specification parameters to become misaligned and overlap details</t>
+  </si>
+  <si>
+    <t>TP1 00:10:58</t>
+  </si>
+  <si>
+    <t>Search for "rx 9060 xt"  → click on a graphics card → Alternatives → Compare all alternatives</t>
+  </si>
+  <si>
+    <t>The user is confused about the meaning of the green number indicators</t>
+  </si>
+  <si>
+    <t>Unclear Meaning of Green Details</t>
+  </si>
+  <si>
+    <t>TP1 00:11:28</t>
+  </si>
+  <si>
+    <t>The user is able to quickly change the website language without any difficulties</t>
+  </si>
+  <si>
+    <t>TP1 00:00:30</t>
+  </si>
+  <si>
+    <t>Homepage</t>
+  </si>
+  <si>
+    <t>The user finds the website easy to navigate for people who are unfamiliar</t>
+  </si>
+  <si>
+    <t>Easy Navigation for New Users</t>
+  </si>
+  <si>
+    <t>Simple Language Switch</t>
+  </si>
+  <si>
+    <t>TP1 00:02:23</t>
   </si>
 </sst>
 </file>
@@ -1182,8 +1106,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
+    <cellStyle name="Link" xfId="1" builtinId="8"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1486,45 +1410,45 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z13"/>
-  <sheetFormatPr defaultColWidth="11.36328125" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.6328125" customWidth="1"/>
-    <col min="2" max="2" width="12.08984375" customWidth="1"/>
-    <col min="3" max="3" width="11.26953125" customWidth="1"/>
-    <col min="4" max="4" width="5.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.6328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" customWidth="1"/>
+    <col min="3" max="3" width="11.28515625" customWidth="1"/>
+    <col min="4" max="4" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="23" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
-    <col min="9" max="9" width="6.7265625" customWidth="1"/>
-    <col min="10" max="10" width="7.81640625" customWidth="1"/>
-    <col min="11" max="11" width="13.6328125" customWidth="1"/>
-    <col min="12" max="12" width="6.26953125" customWidth="1"/>
-    <col min="13" max="13" width="7.08984375" customWidth="1"/>
-    <col min="14" max="14" width="13.6328125" customWidth="1"/>
-    <col min="15" max="15" width="6.26953125" customWidth="1"/>
-    <col min="16" max="16" width="7.6328125" customWidth="1"/>
-    <col min="17" max="17" width="13.36328125" customWidth="1"/>
-    <col min="18" max="18" width="12.7265625" customWidth="1"/>
+    <col min="9" max="9" width="6.7109375" customWidth="1"/>
+    <col min="10" max="10" width="7.85546875" customWidth="1"/>
+    <col min="11" max="11" width="13.5703125" customWidth="1"/>
+    <col min="12" max="12" width="6.28515625" customWidth="1"/>
+    <col min="13" max="13" width="7.140625" customWidth="1"/>
+    <col min="14" max="14" width="13.5703125" customWidth="1"/>
+    <col min="15" max="15" width="6.28515625" customWidth="1"/>
+    <col min="16" max="16" width="7.5703125" customWidth="1"/>
+    <col min="17" max="17" width="13.42578125" customWidth="1"/>
+    <col min="18" max="18" width="12.7109375" customWidth="1"/>
     <col min="19" max="19" width="14" customWidth="1"/>
-    <col min="20" max="20" width="8.26953125" customWidth="1"/>
-    <col min="21" max="21" width="15.26953125" customWidth="1"/>
-    <col min="22" max="22" width="13.453125" customWidth="1"/>
-    <col min="23" max="23" width="13.6328125" customWidth="1"/>
-    <col min="24" max="24" width="13.81640625" customWidth="1"/>
-    <col min="25" max="25" width="13.08984375" customWidth="1"/>
-    <col min="26" max="26" width="22.36328125" customWidth="1"/>
+    <col min="20" max="20" width="8.28515625" customWidth="1"/>
+    <col min="21" max="21" width="15.28515625" customWidth="1"/>
+    <col min="22" max="22" width="13.42578125" customWidth="1"/>
+    <col min="23" max="23" width="13.5703125" customWidth="1"/>
+    <col min="24" max="24" width="13.85546875" customWidth="1"/>
+    <col min="25" max="25" width="13.140625" customWidth="1"/>
+    <col min="26" max="26" width="22.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="2" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:26" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:26" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C3" s="9" t="s">
-        <v>84</v>
+        <v>49</v>
       </c>
       <c r="D3" s="10"/>
       <c r="E3" s="10"/>
@@ -1533,28 +1457,28 @@
       </c>
       <c r="G3" s="11"/>
       <c r="H3" s="9" t="s">
-        <v>91</v>
+        <v>56</v>
       </c>
       <c r="I3" s="10"/>
       <c r="J3" s="10"/>
       <c r="K3" s="9" t="s">
-        <v>90</v>
+        <v>55</v>
       </c>
       <c r="L3" s="10"/>
       <c r="M3" s="10"/>
       <c r="N3" s="9" t="s">
-        <v>99</v>
+        <v>64</v>
       </c>
       <c r="O3" s="10"/>
       <c r="P3" s="10"/>
       <c r="Q3" s="9" t="s">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="R3" s="10"/>
       <c r="S3" s="10"/>
       <c r="T3" s="10"/>
       <c r="U3" s="76" t="s">
-        <v>107</v>
+        <v>72</v>
       </c>
       <c r="V3" s="77"/>
       <c r="W3" s="78"/>
@@ -1564,7 +1488,7 @@
       <c r="Y3" s="78"/>
       <c r="Z3" s="11"/>
     </row>
-    <row r="4" spans="1:26" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:26" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="31" t="s">
         <v>16</v>
       </c>
@@ -1572,7 +1496,7 @@
         <v>6</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>112</v>
+        <v>77</v>
       </c>
       <c r="D4" s="72" t="s">
         <v>7</v>
@@ -1581,40 +1505,40 @@
         <v>8</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>113</v>
+        <v>78</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>135</v>
+        <v>86</v>
       </c>
       <c r="H4" s="12" t="s">
         <v>10</v>
       </c>
       <c r="I4" s="71" t="s">
-        <v>92</v>
+        <v>57</v>
       </c>
       <c r="J4" s="72" t="s">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="K4" s="12" t="s">
         <v>10</v>
       </c>
       <c r="L4" s="71" t="s">
-        <v>92</v>
+        <v>57</v>
       </c>
       <c r="M4" s="72" t="s">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="N4" s="12" t="s">
         <v>10</v>
       </c>
       <c r="O4" s="71" t="s">
-        <v>92</v>
+        <v>57</v>
       </c>
       <c r="P4" s="72" t="s">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="Q4" s="13" t="s">
-        <v>86</v>
+        <v>51</v>
       </c>
       <c r="R4" s="13" t="s">
         <v>12</v>
@@ -1623,36 +1547,36 @@
         <v>0</v>
       </c>
       <c r="T4" s="75" t="s">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="U4" s="13" t="s">
-        <v>139</v>
+        <v>90</v>
       </c>
       <c r="V4" s="13" t="s">
-        <v>138</v>
+        <v>89</v>
       </c>
       <c r="W4" s="13" t="s">
-        <v>140</v>
+        <v>91</v>
       </c>
       <c r="X4" s="13" t="s">
-        <v>108</v>
+        <v>73</v>
       </c>
       <c r="Y4" s="13" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="Z4" s="14" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>17</v>
       </c>
       <c r="B5" s="38" t="s">
-        <v>141</v>
+        <v>92</v>
       </c>
       <c r="C5" s="73" t="s">
-        <v>120</v>
+        <v>85</v>
       </c>
       <c r="D5" s="52">
         <v>19</v>
@@ -1661,10 +1585,10 @@
         <v>15</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>136</v>
+        <v>87</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>146</v>
+        <v>97</v>
       </c>
       <c r="H5" s="41" t="s">
         <v>11</v>
@@ -1676,7 +1600,7 @@
         <v>7</v>
       </c>
       <c r="K5" s="41" t="s">
-        <v>154</v>
+        <v>105</v>
       </c>
       <c r="L5" s="52">
         <v>15</v>
@@ -1685,7 +1609,7 @@
         <v>28</v>
       </c>
       <c r="N5" s="41" t="s">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="O5" s="52">
         <v>10</v>
@@ -1694,45 +1618,45 @@
         <v>28</v>
       </c>
       <c r="Q5" s="42" t="s">
-        <v>87</v>
+        <v>52</v>
       </c>
       <c r="R5" s="16" t="s">
-        <v>102</v>
+        <v>67</v>
       </c>
       <c r="S5" t="s">
-        <v>103</v>
+        <v>68</v>
       </c>
       <c r="T5" s="16">
         <v>4</v>
       </c>
       <c r="U5" s="43" t="s">
-        <v>158</v>
+        <v>109</v>
       </c>
       <c r="V5" s="43" t="s">
-        <v>160</v>
+        <v>111</v>
       </c>
       <c r="W5" s="43" t="s">
-        <v>164</v>
+        <v>115</v>
       </c>
       <c r="X5" s="43" t="s">
-        <v>106</v>
+        <v>71</v>
       </c>
       <c r="Y5" s="43" t="s">
-        <v>106</v>
+        <v>71</v>
       </c>
       <c r="Z5" s="43" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
       <c r="B6" s="38" t="s">
-        <v>142</v>
+        <v>93</v>
       </c>
       <c r="C6" s="73" t="s">
-        <v>120</v>
+        <v>85</v>
       </c>
       <c r="D6" s="52">
         <v>24</v>
@@ -1741,10 +1665,10 @@
         <v>15</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>137</v>
+        <v>88</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>147</v>
+        <v>98</v>
       </c>
       <c r="H6" s="41" t="s">
         <v>11</v>
@@ -1756,7 +1680,7 @@
         <v>35</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>154</v>
+        <v>105</v>
       </c>
       <c r="L6" s="52">
         <v>15</v>
@@ -1765,7 +1689,7 @@
         <v>25</v>
       </c>
       <c r="N6" s="15" t="s">
-        <v>154</v>
+        <v>105</v>
       </c>
       <c r="O6" s="52">
         <v>12</v>
@@ -1774,45 +1698,45 @@
         <v>25</v>
       </c>
       <c r="Q6" t="s">
-        <v>88</v>
+        <v>53</v>
       </c>
       <c r="R6" s="4" t="s">
-        <v>102</v>
+        <v>67</v>
       </c>
       <c r="S6" s="4" t="s">
-        <v>103</v>
+        <v>68</v>
       </c>
       <c r="T6" s="4">
         <v>15</v>
       </c>
       <c r="U6" s="43" t="s">
-        <v>158</v>
+        <v>109</v>
       </c>
       <c r="V6" s="4" t="s">
-        <v>160</v>
+        <v>111</v>
       </c>
       <c r="W6" s="4" t="s">
-        <v>164</v>
+        <v>115</v>
       </c>
       <c r="X6" s="43" t="s">
-        <v>106</v>
+        <v>71</v>
       </c>
       <c r="Y6" s="4" t="s">
-        <v>106</v>
+        <v>71</v>
       </c>
       <c r="Z6" s="43" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B7" s="38" t="s">
-        <v>143</v>
+        <v>94</v>
       </c>
       <c r="C7" s="73" t="s">
-        <v>120</v>
+        <v>85</v>
       </c>
       <c r="D7" s="52">
         <v>19</v>
@@ -1821,10 +1745,10 @@
         <v>15</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>152</v>
+        <v>103</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>148</v>
+        <v>99</v>
       </c>
       <c r="H7" s="15" t="s">
         <v>11</v>
@@ -1833,10 +1757,10 @@
         <v>8</v>
       </c>
       <c r="J7" s="52" t="s">
-        <v>153</v>
+        <v>104</v>
       </c>
       <c r="K7" s="15" t="s">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="L7" s="52">
         <v>30</v>
@@ -1845,7 +1769,7 @@
         <v>60</v>
       </c>
       <c r="N7" s="15" t="s">
-        <v>154</v>
+        <v>105</v>
       </c>
       <c r="O7" s="52">
         <v>12</v>
@@ -1854,45 +1778,45 @@
         <v>60</v>
       </c>
       <c r="Q7" t="s">
-        <v>89</v>
+        <v>54</v>
       </c>
       <c r="R7" s="4" t="s">
-        <v>155</v>
+        <v>106</v>
       </c>
       <c r="S7" s="4" t="s">
-        <v>103</v>
+        <v>68</v>
       </c>
       <c r="T7" s="4">
         <v>20</v>
       </c>
       <c r="U7" s="43" t="s">
-        <v>158</v>
+        <v>109</v>
       </c>
       <c r="V7" s="4" t="s">
-        <v>161</v>
+        <v>112</v>
       </c>
       <c r="W7" s="4" t="s">
-        <v>164</v>
+        <v>115</v>
       </c>
       <c r="X7" s="43" t="s">
-        <v>106</v>
+        <v>71</v>
       </c>
       <c r="Y7" s="4" t="s">
-        <v>106</v>
+        <v>71</v>
       </c>
       <c r="Z7" s="43" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B8" s="38" t="s">
-        <v>144</v>
+        <v>95</v>
       </c>
       <c r="C8" s="73" t="s">
-        <v>119</v>
+        <v>84</v>
       </c>
       <c r="D8" s="52">
         <v>29</v>
@@ -1901,10 +1825,10 @@
         <v>15</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>152</v>
+        <v>103</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>149</v>
+        <v>100</v>
       </c>
       <c r="H8" s="15" t="s">
         <v>11</v>
@@ -1916,7 +1840,7 @@
         <v>55</v>
       </c>
       <c r="K8" s="15" t="s">
-        <v>94</v>
+        <v>59</v>
       </c>
       <c r="L8" s="52">
         <v>0</v>
@@ -1925,7 +1849,7 @@
         <v>21</v>
       </c>
       <c r="N8" s="15" t="s">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="O8" s="52">
         <v>14</v>
@@ -1934,10 +1858,10 @@
         <v>21</v>
       </c>
       <c r="Q8" t="s">
-        <v>88</v>
+        <v>53</v>
       </c>
       <c r="R8" s="4" t="s">
-        <v>102</v>
+        <v>67</v>
       </c>
       <c r="S8" s="4" t="s">
         <v>1</v>
@@ -1946,33 +1870,33 @@
         <v>30</v>
       </c>
       <c r="U8" s="43" t="s">
-        <v>158</v>
+        <v>109</v>
       </c>
       <c r="V8" s="4" t="s">
-        <v>162</v>
+        <v>113</v>
       </c>
       <c r="W8" s="4" t="s">
-        <v>164</v>
+        <v>115</v>
       </c>
       <c r="X8" s="43" t="s">
-        <v>106</v>
+        <v>71</v>
       </c>
       <c r="Y8" s="4" t="s">
-        <v>106</v>
+        <v>71</v>
       </c>
       <c r="Z8" s="43" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A9" s="19" t="s">
         <v>21</v>
       </c>
       <c r="B9" s="62" t="s">
-        <v>145</v>
+        <v>96</v>
       </c>
       <c r="C9" s="74" t="s">
-        <v>119</v>
+        <v>84</v>
       </c>
       <c r="D9" s="53">
         <v>24</v>
@@ -1981,13 +1905,13 @@
         <v>15</v>
       </c>
       <c r="F9" s="20" t="s">
-        <v>137</v>
+        <v>88</v>
       </c>
       <c r="G9" s="20" t="s">
-        <v>150</v>
+        <v>101</v>
       </c>
       <c r="H9" s="21" t="s">
-        <v>151</v>
+        <v>102</v>
       </c>
       <c r="I9" s="54">
         <v>15</v>
@@ -1996,7 +1920,7 @@
         <v>56</v>
       </c>
       <c r="K9" s="21" t="s">
-        <v>94</v>
+        <v>59</v>
       </c>
       <c r="L9" s="54">
         <v>0</v>
@@ -2005,7 +1929,7 @@
         <v>14</v>
       </c>
       <c r="N9" s="21" t="s">
-        <v>154</v>
+        <v>105</v>
       </c>
       <c r="O9" s="54">
         <v>12</v>
@@ -2014,37 +1938,37 @@
         <v>14</v>
       </c>
       <c r="Q9" s="22" t="s">
-        <v>88</v>
+        <v>53</v>
       </c>
       <c r="R9" s="20" t="s">
-        <v>156</v>
+        <v>107</v>
       </c>
       <c r="S9" s="22" t="s">
-        <v>157</v>
+        <v>108</v>
       </c>
       <c r="T9" s="20">
         <v>28</v>
       </c>
       <c r="U9" s="20" t="s">
-        <v>159</v>
+        <v>110</v>
       </c>
       <c r="V9" s="20" t="s">
-        <v>163</v>
+        <v>114</v>
       </c>
       <c r="W9" s="20" t="s">
-        <v>164</v>
+        <v>115</v>
       </c>
       <c r="X9" s="61" t="s">
-        <v>106</v>
+        <v>71</v>
       </c>
       <c r="Y9" s="20" t="s">
-        <v>106</v>
+        <v>71</v>
       </c>
       <c r="Z9" s="43" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="10" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="I10" s="18"/>
       <c r="J10" s="18"/>
       <c r="L10" s="18"/>
@@ -2052,10 +1976,10 @@
       <c r="O10" s="18"/>
       <c r="P10" s="18"/>
     </row>
-    <row r="11" spans="1:26" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A11" s="24"/>
       <c r="B11" s="26" t="s">
-        <v>78</v>
+        <v>43</v>
       </c>
       <c r="C11" s="5"/>
       <c r="D11" s="51">
@@ -2066,7 +1990,7 @@
       <c r="F11" s="17"/>
       <c r="G11" s="17"/>
       <c r="H11" s="40" t="s">
-        <v>116</v>
+        <v>81</v>
       </c>
       <c r="I11" s="45">
         <f>AVERAGE(I5:I9)</f>
@@ -2077,7 +2001,7 @@
         <v>38.25</v>
       </c>
       <c r="K11" s="40" t="s">
-        <v>95</v>
+        <v>60</v>
       </c>
       <c r="L11" s="45">
         <f>AVERAGE(L5:L9)</f>
@@ -2088,7 +2012,7 @@
         <v>29.6</v>
       </c>
       <c r="N11" s="40" t="s">
-        <v>101</v>
+        <v>66</v>
       </c>
       <c r="O11" s="45">
         <f>AVERAGE(O5:O9)</f>
@@ -2101,14 +2025,14 @@
       <c r="Q11" s="17"/>
       <c r="R11" s="17"/>
       <c r="S11" s="40" t="s">
-        <v>104</v>
+        <v>69</v>
       </c>
       <c r="T11" s="45">
         <f>AVERAGE(T5:T9)</f>
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="24"/>
       <c r="B12" s="26" t="s">
         <v>14</v>
@@ -2119,7 +2043,7 @@
         <v>24</v>
       </c>
       <c r="H12" t="s">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="I12" s="28">
         <f>MEDIAN(I5:I9)</f>
@@ -2130,7 +2054,7 @@
         <v>45</v>
       </c>
       <c r="K12" t="s">
-        <v>96</v>
+        <v>61</v>
       </c>
       <c r="L12" s="28">
         <f>MEDIAN(L5:L9)</f>
@@ -2141,7 +2065,7 @@
         <v>25</v>
       </c>
       <c r="N12" t="s">
-        <v>95</v>
+        <v>60</v>
       </c>
       <c r="O12" s="28">
         <f>MEDIAN(O5:O9)</f>
@@ -2152,22 +2076,22 @@
         <v>25</v>
       </c>
       <c r="S12" s="40" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="T12" s="28">
         <f>MEDIAN(T5:T9)</f>
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.2">
       <c r="H13" t="s">
-        <v>97</v>
+        <v>62</v>
       </c>
       <c r="K13" t="s">
-        <v>98</v>
+        <v>63</v>
       </c>
       <c r="S13" s="40" t="s">
-        <v>114</v>
+        <v>79</v>
       </c>
       <c r="T13" s="40"/>
     </row>
@@ -2186,22 +2110,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultColWidth="11.36328125" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.08984375" style="23" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7265625" customWidth="1"/>
-    <col min="4" max="4" width="15.7265625" customWidth="1"/>
-    <col min="5" max="5" width="11.7265625" customWidth="1"/>
-    <col min="6" max="7" width="10.7265625" customWidth="1"/>
+    <col min="1" max="1" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" style="23" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" customWidth="1"/>
+    <col min="6" max="7" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="13" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C3" s="35" t="s">
         <v>4</v>
       </c>
@@ -2210,7 +2134,7 @@
       <c r="F3" s="25"/>
       <c r="G3" s="25"/>
     </row>
-    <row r="4" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="31" t="s">
         <v>16</v>
       </c>
@@ -2221,24 +2145,24 @@
         <v>22</v>
       </c>
       <c r="D4" s="25" t="s">
-        <v>166</v>
+        <v>117</v>
       </c>
       <c r="E4" s="25" t="s">
-        <v>167</v>
+        <v>118</v>
       </c>
       <c r="F4" s="25" t="s">
-        <v>168</v>
+        <v>119</v>
       </c>
       <c r="G4" s="25" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>17</v>
       </c>
       <c r="B5" s="38" t="s">
-        <v>141</v>
+        <v>92</v>
       </c>
       <c r="C5" s="27">
         <v>1</v>
@@ -2256,12 +2180,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
       <c r="B6" s="38" t="s">
-        <v>142</v>
+        <v>93</v>
       </c>
       <c r="C6" s="27">
         <v>1</v>
@@ -2279,12 +2203,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B7" s="38" t="s">
-        <v>143</v>
+        <v>94</v>
       </c>
       <c r="C7" s="27">
         <v>1</v>
@@ -2302,12 +2226,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B8" s="38" t="s">
-        <v>144</v>
+        <v>95</v>
       </c>
       <c r="C8" s="27">
         <v>1</v>
@@ -2325,12 +2249,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
         <v>21</v>
       </c>
       <c r="B9" s="62" t="s">
-        <v>145</v>
+        <v>96</v>
       </c>
       <c r="C9" s="27">
         <v>1</v>
@@ -2348,7 +2272,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="24"/>
       <c r="B10" s="24" t="s">
         <v>2</v>
@@ -2374,7 +2298,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="24"/>
       <c r="B11" s="24" t="s">
         <v>3</v>
@@ -2411,29 +2335,29 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K14"/>
-  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
-    <col min="2" max="2" width="36.08984375" customWidth="1"/>
-    <col min="3" max="3" width="35.08984375" customWidth="1"/>
-    <col min="4" max="4" width="34.453125" customWidth="1"/>
-    <col min="5" max="5" width="25.81640625" customWidth="1"/>
+    <col min="2" max="2" width="36.140625" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" customWidth="1"/>
+    <col min="4" max="4" width="34.42578125" customWidth="1"/>
+    <col min="5" max="5" width="25.85546875" customWidth="1"/>
     <col min="6" max="6" width="29" customWidth="1"/>
-    <col min="7" max="10" width="4.6328125" style="55" customWidth="1"/>
-    <col min="11" max="11" width="6.08984375" style="55" customWidth="1"/>
+    <col min="7" max="10" width="4.5703125" style="55" customWidth="1"/>
+    <col min="11" max="11" width="6.140625" style="55" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="G3" s="58" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:11" s="56" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" s="56" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="60" t="s">
         <v>32</v>
       </c>
@@ -2444,429 +2368,251 @@
         <v>34</v>
       </c>
       <c r="D4" s="60" t="s">
-        <v>111</v>
+        <v>76</v>
       </c>
       <c r="E4" s="60" t="s">
         <v>35</v>
       </c>
       <c r="F4" s="60" t="s">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="G4" s="57" t="s">
-        <v>49</v>
+        <v>124</v>
       </c>
       <c r="H4" s="57" t="s">
-        <v>50</v>
+        <v>125</v>
       </c>
       <c r="I4" s="57" t="s">
-        <v>51</v>
+        <v>126</v>
       </c>
       <c r="J4" s="57" t="s">
-        <v>52</v>
+        <v>127</v>
       </c>
       <c r="K4" s="59" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="25" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A5" s="63">
         <v>1</v>
       </c>
       <c r="B5" s="64" t="s">
+        <v>122</v>
+      </c>
+      <c r="C5" s="69" t="s">
+        <v>121</v>
+      </c>
+      <c r="D5" s="69"/>
+      <c r="E5" s="69" t="s">
+        <v>123</v>
+      </c>
+      <c r="F5" s="69" t="s">
         <v>128</v>
       </c>
-      <c r="C5" s="69" t="s">
+      <c r="G5" s="66"/>
+      <c r="H5" s="66"/>
+      <c r="I5" s="66"/>
+      <c r="J5" s="66">
+        <v>2</v>
+      </c>
+      <c r="K5" s="67">
+        <f>AVERAGE(G5:J5)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A6" s="63">
+        <v>2</v>
+      </c>
+      <c r="B6" s="64" t="s">
+        <v>130</v>
+      </c>
+      <c r="C6" s="64" t="s">
         <v>129</v>
       </c>
-      <c r="D5" s="69" t="s">
+      <c r="D6" s="63"/>
+      <c r="E6" s="63" t="s">
+        <v>131</v>
+      </c>
+      <c r="F6" s="69" t="s">
         <v>132</v>
       </c>
-      <c r="E5" s="69" t="s">
+      <c r="G6" s="66"/>
+      <c r="H6" s="66"/>
+      <c r="I6" s="66"/>
+      <c r="J6" s="66">
+        <v>2</v>
+      </c>
+      <c r="K6" s="67">
+        <f>AVERAGE(G6:J6)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A7" s="63">
+        <v>3</v>
+      </c>
+      <c r="B7" s="64" t="s">
         <v>133</v>
       </c>
-      <c r="F5" s="69" t="s">
-        <v>121</v>
-      </c>
-      <c r="G5" s="66">
-        <v>2</v>
-      </c>
-      <c r="H5" s="66">
+      <c r="C7" s="64" t="s">
+        <v>134</v>
+      </c>
+      <c r="D7" s="63"/>
+      <c r="E7" s="63" t="s">
+        <v>135</v>
+      </c>
+      <c r="F7" s="64" t="s">
+        <v>136</v>
+      </c>
+      <c r="G7" s="66"/>
+      <c r="H7" s="66"/>
+      <c r="I7" s="66"/>
+      <c r="J7" s="66">
+        <v>3</v>
+      </c>
+      <c r="K7" s="67">
+        <f>AVERAGE(G7:J7)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A8" s="63">
         <v>4</v>
       </c>
-      <c r="I5" s="66">
-        <v>4</v>
-      </c>
-      <c r="J5" s="66">
-        <v>4</v>
-      </c>
-      <c r="K5" s="67">
-        <f t="shared" ref="K5:K14" si="0">AVERAGE(G5:J5)</f>
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="25" x14ac:dyDescent="0.25">
-      <c r="A6" s="63">
-        <f>SUM(A5,1)</f>
-        <v>2</v>
-      </c>
-      <c r="B6" s="64" t="s">
-        <v>60</v>
-      </c>
-      <c r="C6" s="64" t="s">
-        <v>61</v>
-      </c>
-      <c r="D6" s="63" t="s">
-        <v>76</v>
-      </c>
-      <c r="E6" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="F6" s="69" t="s">
-        <v>123</v>
-      </c>
-      <c r="G6" s="66">
-        <v>3</v>
-      </c>
-      <c r="H6" s="66">
-        <v>4</v>
-      </c>
-      <c r="I6" s="66">
-        <v>3</v>
-      </c>
-      <c r="J6" s="66">
-        <v>3</v>
-      </c>
-      <c r="K6" s="67">
-        <f t="shared" si="0"/>
-        <v>3.25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="63">
-        <f>SUM(A6,1)</f>
-        <v>3</v>
-      </c>
-      <c r="B7" s="64" t="s">
-        <v>36</v>
-      </c>
-      <c r="C7" s="64" t="s">
-        <v>37</v>
-      </c>
-      <c r="D7" s="63" t="s">
-        <v>69</v>
-      </c>
-      <c r="E7" s="63" t="s">
-        <v>55</v>
-      </c>
-      <c r="F7" s="64" t="s">
-        <v>38</v>
-      </c>
-      <c r="G7" s="66">
-        <v>4</v>
-      </c>
-      <c r="H7" s="66">
-        <v>2</v>
-      </c>
-      <c r="I7" s="66">
-        <v>3</v>
-      </c>
-      <c r="J7" s="66">
-        <v>4</v>
-      </c>
-      <c r="K7" s="67">
-        <f t="shared" si="0"/>
-        <v>3.25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="25" x14ac:dyDescent="0.25">
-      <c r="A8" s="63">
-        <f>SUM(A7,1)</f>
-        <v>4</v>
-      </c>
       <c r="B8" s="64" t="s">
-        <v>39</v>
+        <v>138</v>
       </c>
       <c r="C8" s="64" t="s">
-        <v>40</v>
-      </c>
-      <c r="D8" s="63" t="s">
-        <v>69</v>
-      </c>
+        <v>137</v>
+      </c>
+      <c r="D8" s="63"/>
       <c r="E8" s="69" t="s">
-        <v>134</v>
-      </c>
-      <c r="F8" s="70" t="s">
-        <v>125</v>
-      </c>
-      <c r="G8" s="66">
-        <v>3</v>
-      </c>
-      <c r="H8" s="66">
-        <v>3</v>
-      </c>
-      <c r="I8" s="66">
-        <v>3</v>
-      </c>
+        <v>139</v>
+      </c>
+      <c r="F8" s="64" t="s">
+        <v>136</v>
+      </c>
+      <c r="G8" s="66"/>
+      <c r="H8" s="66"/>
+      <c r="I8" s="66"/>
       <c r="J8" s="66">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K8" s="67">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="63">
-        <f>SUM(A8,1)</f>
-        <v>5</v>
-      </c>
-      <c r="B9" s="64" t="s">
-        <v>41</v>
-      </c>
-      <c r="C9" s="64" t="s">
-        <v>42</v>
-      </c>
-      <c r="D9" s="63" t="s">
-        <v>69</v>
-      </c>
-      <c r="E9" s="63" t="s">
-        <v>57</v>
-      </c>
-      <c r="F9" s="69" t="s">
-        <v>124</v>
-      </c>
-      <c r="G9" s="66">
-        <v>3</v>
-      </c>
-      <c r="H9" s="66">
-        <v>2</v>
-      </c>
-      <c r="I9" s="66">
-        <v>2</v>
-      </c>
-      <c r="J9" s="66">
-        <v>3</v>
-      </c>
-      <c r="K9" s="67">
-        <f t="shared" si="0"/>
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="25" x14ac:dyDescent="0.25">
-      <c r="A10" s="63">
-        <v>6</v>
-      </c>
-      <c r="B10" s="64" t="s">
-        <v>43</v>
-      </c>
-      <c r="C10" s="64" t="s">
-        <v>44</v>
-      </c>
-      <c r="D10" s="63" t="s">
-        <v>69</v>
-      </c>
-      <c r="E10" s="63" t="s">
-        <v>58</v>
-      </c>
-      <c r="F10" s="69" t="s">
-        <v>122</v>
-      </c>
-      <c r="G10" s="66">
-        <v>2</v>
-      </c>
-      <c r="H10" s="66">
-        <v>2</v>
-      </c>
-      <c r="I10" s="66">
-        <v>2</v>
-      </c>
-      <c r="J10" s="66">
-        <v>2</v>
-      </c>
-      <c r="K10" s="67">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="25" x14ac:dyDescent="0.25">
-      <c r="A11" s="63">
-        <v>7</v>
-      </c>
-      <c r="B11" s="64" t="s">
-        <v>45</v>
-      </c>
-      <c r="C11" s="64" t="s">
-        <v>46</v>
-      </c>
-      <c r="D11" s="63" t="s">
-        <v>69</v>
-      </c>
-      <c r="E11" s="63" t="s">
-        <v>59</v>
-      </c>
-      <c r="F11" s="64" t="s">
-        <v>47</v>
-      </c>
-      <c r="G11" s="66">
-        <v>2</v>
-      </c>
-      <c r="H11" s="66">
-        <v>2</v>
-      </c>
-      <c r="I11" s="66">
-        <v>2</v>
-      </c>
-      <c r="J11" s="66">
-        <v>2</v>
-      </c>
-      <c r="K11" s="67">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="68" t="s">
-        <v>69</v>
-      </c>
-      <c r="B12" s="69" t="s">
-        <v>69</v>
-      </c>
-      <c r="C12" s="69" t="s">
-        <v>69</v>
-      </c>
-      <c r="D12" s="65" t="s">
-        <v>69</v>
-      </c>
-      <c r="E12" s="65" t="s">
-        <v>69</v>
-      </c>
-      <c r="F12" s="69" t="s">
-        <v>69</v>
-      </c>
-      <c r="G12" s="66">
-        <v>2</v>
-      </c>
-      <c r="H12" s="66">
+        <f>AVERAGE(G8:J8)</f>
         <v>1</v>
       </c>
-      <c r="I12" s="66">
-        <v>1</v>
-      </c>
-      <c r="J12" s="66">
-        <v>3</v>
-      </c>
-      <c r="K12" s="67">
-        <f t="shared" si="0"/>
-        <v>1.75</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="68" t="s">
-        <v>69</v>
-      </c>
-      <c r="B13" s="69" t="s">
-        <v>69</v>
-      </c>
-      <c r="C13" s="69" t="s">
-        <v>69</v>
-      </c>
-      <c r="D13" s="65" t="s">
-        <v>69</v>
-      </c>
-      <c r="E13" s="65" t="s">
-        <v>69</v>
-      </c>
-      <c r="F13" s="69" t="s">
-        <v>69</v>
-      </c>
-      <c r="G13" s="66">
-        <v>2</v>
-      </c>
-      <c r="H13" s="66">
-        <v>1</v>
-      </c>
-      <c r="I13" s="66">
-        <v>1</v>
-      </c>
-      <c r="J13" s="66">
-        <v>1</v>
-      </c>
-      <c r="K13" s="67">
-        <f t="shared" si="0"/>
-        <v>1.25</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="25" x14ac:dyDescent="0.25">
-      <c r="A14" s="63">
-        <v>21</v>
-      </c>
-      <c r="B14" s="64" t="s">
-        <v>48</v>
-      </c>
-      <c r="C14" s="64" t="s">
-        <v>53</v>
-      </c>
-      <c r="D14" s="65" t="s">
-        <v>77</v>
-      </c>
-      <c r="E14" s="65" t="s">
-        <v>74</v>
-      </c>
-      <c r="F14" s="70" t="s">
-        <v>125</v>
-      </c>
-      <c r="G14" s="66">
-        <v>1</v>
-      </c>
-      <c r="H14" s="66">
-        <v>0</v>
-      </c>
-      <c r="I14" s="66">
-        <v>1</v>
-      </c>
-      <c r="J14" s="66">
-        <v>1</v>
-      </c>
-      <c r="K14" s="67">
-        <f t="shared" si="0"/>
-        <v>0.75</v>
-      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" s="63"/>
+      <c r="B9" s="64"/>
+      <c r="C9" s="64"/>
+      <c r="D9" s="63"/>
+      <c r="E9" s="63"/>
+      <c r="F9" s="69"/>
+      <c r="G9" s="66"/>
+      <c r="H9" s="66"/>
+      <c r="I9" s="66"/>
+      <c r="J9" s="66"/>
+      <c r="K9" s="67"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" s="63"/>
+      <c r="B10" s="64"/>
+      <c r="C10" s="64"/>
+      <c r="D10" s="63"/>
+      <c r="E10" s="63"/>
+      <c r="F10" s="69"/>
+      <c r="G10" s="66"/>
+      <c r="H10" s="66"/>
+      <c r="I10" s="66"/>
+      <c r="J10" s="66"/>
+      <c r="K10" s="67"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11" s="63"/>
+      <c r="B11" s="64"/>
+      <c r="C11" s="64"/>
+      <c r="D11" s="63"/>
+      <c r="E11" s="63"/>
+      <c r="F11" s="64"/>
+      <c r="G11" s="66"/>
+      <c r="H11" s="66"/>
+      <c r="I11" s="66"/>
+      <c r="J11" s="66"/>
+      <c r="K11" s="67"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12" s="68"/>
+      <c r="B12" s="69"/>
+      <c r="C12" s="69"/>
+      <c r="D12" s="65"/>
+      <c r="E12" s="65"/>
+      <c r="F12" s="69"/>
+      <c r="G12" s="66"/>
+      <c r="H12" s="66"/>
+      <c r="I12" s="66"/>
+      <c r="J12" s="66"/>
+      <c r="K12" s="67"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" s="68"/>
+      <c r="B13" s="69"/>
+      <c r="C13" s="69"/>
+      <c r="D13" s="65"/>
+      <c r="E13" s="65"/>
+      <c r="F13" s="69"/>
+      <c r="G13" s="66"/>
+      <c r="H13" s="66"/>
+      <c r="I13" s="66"/>
+      <c r="J13" s="66"/>
+      <c r="K13" s="67"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A14" s="63"/>
+      <c r="B14" s="64"/>
+      <c r="C14" s="64"/>
+      <c r="D14" s="65"/>
+      <c r="E14" s="65"/>
+      <c r="F14" s="70"/>
+      <c r="G14" s="66"/>
+      <c r="H14" s="66"/>
+      <c r="I14" s="66"/>
+      <c r="J14" s="66"/>
+      <c r="K14" s="67"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="F8" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
-    <hyperlink ref="F14" r:id="rId2" xr:uid="{00000000-0004-0000-0200-000001000000}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K14"/>
-  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
-    <col min="3" max="4" width="35.08984375" customWidth="1"/>
-    <col min="5" max="5" width="26.08984375" customWidth="1"/>
-    <col min="6" max="6" width="29.08984375" customWidth="1"/>
-    <col min="7" max="10" width="4.6328125" style="55" customWidth="1"/>
-    <col min="11" max="11" width="5.81640625" style="55" customWidth="1"/>
+    <col min="3" max="4" width="35.140625" customWidth="1"/>
+    <col min="5" max="5" width="26.140625" customWidth="1"/>
+    <col min="6" max="6" width="29.140625" customWidth="1"/>
+    <col min="7" max="10" width="4.5703125" style="55" customWidth="1"/>
+    <col min="11" max="11" width="5.85546875" style="55" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="G3" s="58" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" s="56" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" s="56" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="60" t="s">
         <v>32</v>
       </c>
@@ -2877,393 +2623,189 @@
         <v>34</v>
       </c>
       <c r="D4" s="60" t="s">
-        <v>111</v>
+        <v>76</v>
       </c>
       <c r="E4" s="60" t="s">
         <v>35</v>
       </c>
       <c r="F4" s="60" t="s">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="G4" s="57" t="s">
-        <v>49</v>
+        <v>124</v>
       </c>
       <c r="H4" s="57" t="s">
-        <v>50</v>
+        <v>125</v>
       </c>
       <c r="I4" s="57" t="s">
-        <v>51</v>
+        <v>126</v>
       </c>
       <c r="J4" s="57" t="s">
-        <v>52</v>
+        <v>127</v>
       </c>
       <c r="K4" s="59" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="37.5" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A5" s="63">
         <v>1</v>
       </c>
       <c r="B5" s="64" t="s">
-        <v>70</v>
+        <v>145</v>
       </c>
       <c r="C5" s="64" t="s">
-        <v>71</v>
-      </c>
-      <c r="D5" s="69" t="s">
-        <v>130</v>
-      </c>
+        <v>140</v>
+      </c>
+      <c r="D5" s="69"/>
       <c r="E5" s="69" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="F5" s="69" t="s">
-        <v>126</v>
-      </c>
-      <c r="G5" s="66">
+        <v>142</v>
+      </c>
+      <c r="G5" s="66"/>
+      <c r="H5" s="66"/>
+      <c r="I5" s="66"/>
+      <c r="J5" s="66">
+        <v>1</v>
+      </c>
+      <c r="K5" s="67">
+        <f>AVERAGE(G5:J5)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A6" s="63">
         <v>2</v>
       </c>
-      <c r="H5" s="66">
-        <v>4</v>
-      </c>
-      <c r="I5" s="66">
-        <v>4</v>
-      </c>
-      <c r="J5" s="66">
-        <v>4</v>
-      </c>
-      <c r="K5" s="67">
-        <f t="shared" ref="K5:K14" si="0">AVERAGE(G5:J5)</f>
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="63">
-        <f>SUM(A5,1)</f>
+      <c r="B6" s="64" t="s">
+        <v>144</v>
+      </c>
+      <c r="C6" s="64" t="s">
+        <v>143</v>
+      </c>
+      <c r="D6" s="64"/>
+      <c r="E6" s="64" t="s">
+        <v>146</v>
+      </c>
+      <c r="F6" s="69" t="s">
+        <v>142</v>
+      </c>
+      <c r="G6" s="66"/>
+      <c r="H6" s="66"/>
+      <c r="I6" s="66"/>
+      <c r="J6" s="66">
         <v>2</v>
       </c>
-      <c r="B6" s="64" t="s">
-        <v>73</v>
-      </c>
-      <c r="C6" s="64" t="s">
-        <v>72</v>
-      </c>
-      <c r="D6" s="64" t="s">
-        <v>75</v>
-      </c>
-      <c r="E6" s="64" t="s">
-        <v>54</v>
-      </c>
-      <c r="F6" s="69" t="s">
-        <v>127</v>
-      </c>
-      <c r="G6" s="66">
-        <v>3</v>
-      </c>
-      <c r="H6" s="66">
-        <v>4</v>
-      </c>
-      <c r="I6" s="66">
-        <v>3</v>
-      </c>
-      <c r="J6" s="66">
-        <v>3</v>
-      </c>
       <c r="K6" s="67">
-        <f t="shared" si="0"/>
-        <v>3.25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="63">
-        <f>SUM(A6,1)</f>
-        <v>3</v>
-      </c>
-      <c r="B7" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="C7" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="D7" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="E7" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="F7" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="G7" s="66">
-        <v>4</v>
-      </c>
-      <c r="H7" s="66">
+        <f>AVERAGE(G6:J6)</f>
         <v>2</v>
       </c>
-      <c r="I7" s="66">
-        <v>3</v>
-      </c>
-      <c r="J7" s="66">
-        <v>4</v>
-      </c>
-      <c r="K7" s="67">
-        <f t="shared" si="0"/>
-        <v>3.25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="63">
-        <f>SUM(A7,1)</f>
-        <v>4</v>
-      </c>
-      <c r="B8" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="C8" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="D8" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="E8" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="F8" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="G8" s="66">
-        <v>3</v>
-      </c>
-      <c r="H8" s="66">
-        <v>3</v>
-      </c>
-      <c r="I8" s="66">
-        <v>3</v>
-      </c>
-      <c r="J8" s="66">
-        <v>3</v>
-      </c>
-      <c r="K8" s="67">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="63">
-        <f>SUM(A8,1)</f>
-        <v>5</v>
-      </c>
-      <c r="B9" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="C9" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="D9" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="E9" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="F9" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="G9" s="66">
-        <v>3</v>
-      </c>
-      <c r="H9" s="66">
-        <v>2</v>
-      </c>
-      <c r="I9" s="66">
-        <v>2</v>
-      </c>
-      <c r="J9" s="66">
-        <v>3</v>
-      </c>
-      <c r="K9" s="67">
-        <f t="shared" si="0"/>
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="63">
-        <v>6</v>
-      </c>
-      <c r="B10" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="C10" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="D10" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="E10" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="F10" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="G10" s="66">
-        <v>2</v>
-      </c>
-      <c r="H10" s="66">
-        <v>2</v>
-      </c>
-      <c r="I10" s="66">
-        <v>2</v>
-      </c>
-      <c r="J10" s="66">
-        <v>2</v>
-      </c>
-      <c r="K10" s="67">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="63">
-        <v>7</v>
-      </c>
-      <c r="B11" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="C11" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="D11" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="E11" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="F11" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="G11" s="66">
-        <v>2</v>
-      </c>
-      <c r="H11" s="66">
-        <v>2</v>
-      </c>
-      <c r="I11" s="66">
-        <v>2</v>
-      </c>
-      <c r="J11" s="66">
-        <v>2</v>
-      </c>
-      <c r="K11" s="67">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="63">
-        <v>8</v>
-      </c>
-      <c r="B12" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="C12" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="D12" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="E12" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="F12" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="G12" s="66">
-        <v>2</v>
-      </c>
-      <c r="H12" s="66">
-        <v>1</v>
-      </c>
-      <c r="I12" s="66">
-        <v>1</v>
-      </c>
-      <c r="J12" s="66">
-        <v>3</v>
-      </c>
-      <c r="K12" s="67">
-        <f t="shared" si="0"/>
-        <v>1.75</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="63">
-        <v>9</v>
-      </c>
-      <c r="B13" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="C13" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="D13" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="E13" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="F13" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="G13" s="66">
-        <v>2</v>
-      </c>
-      <c r="H13" s="66">
-        <v>1</v>
-      </c>
-      <c r="I13" s="66">
-        <v>1</v>
-      </c>
-      <c r="J13" s="66">
-        <v>1</v>
-      </c>
-      <c r="K13" s="67">
-        <f t="shared" si="0"/>
-        <v>1.25</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="63">
-        <v>10</v>
-      </c>
-      <c r="B14" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="C14" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="D14" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="E14" s="64" t="s">
-        <v>56</v>
-      </c>
-      <c r="F14" s="64" t="s">
-        <v>69</v>
-      </c>
-      <c r="G14" s="66">
-        <v>1</v>
-      </c>
-      <c r="H14" s="66">
-        <v>0</v>
-      </c>
-      <c r="I14" s="66">
-        <v>1</v>
-      </c>
-      <c r="J14" s="66">
-        <v>1</v>
-      </c>
-      <c r="K14" s="67">
-        <f t="shared" si="0"/>
-        <v>0.75</v>
-      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7" s="63"/>
+      <c r="B7" s="64"/>
+      <c r="C7" s="64"/>
+      <c r="D7" s="64"/>
+      <c r="E7" s="64"/>
+      <c r="F7" s="64"/>
+      <c r="G7" s="66"/>
+      <c r="H7" s="66"/>
+      <c r="I7" s="66"/>
+      <c r="J7" s="66"/>
+      <c r="K7" s="67"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8" s="63"/>
+      <c r="B8" s="64"/>
+      <c r="C8" s="64"/>
+      <c r="D8" s="64"/>
+      <c r="E8" s="64"/>
+      <c r="F8" s="64"/>
+      <c r="G8" s="66"/>
+      <c r="H8" s="66"/>
+      <c r="I8" s="66"/>
+      <c r="J8" s="66"/>
+      <c r="K8" s="67"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" s="63"/>
+      <c r="B9" s="64"/>
+      <c r="C9" s="64"/>
+      <c r="D9" s="64"/>
+      <c r="E9" s="64"/>
+      <c r="F9" s="64"/>
+      <c r="G9" s="66"/>
+      <c r="H9" s="66"/>
+      <c r="I9" s="66"/>
+      <c r="J9" s="66"/>
+      <c r="K9" s="67"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" s="63"/>
+      <c r="B10" s="64"/>
+      <c r="C10" s="64"/>
+      <c r="D10" s="64"/>
+      <c r="E10" s="64"/>
+      <c r="F10" s="64"/>
+      <c r="G10" s="66"/>
+      <c r="H10" s="66"/>
+      <c r="I10" s="66"/>
+      <c r="J10" s="66"/>
+      <c r="K10" s="67"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11" s="63"/>
+      <c r="B11" s="64"/>
+      <c r="C11" s="64"/>
+      <c r="D11" s="64"/>
+      <c r="E11" s="64"/>
+      <c r="F11" s="64"/>
+      <c r="G11" s="66"/>
+      <c r="H11" s="66"/>
+      <c r="I11" s="66"/>
+      <c r="J11" s="66"/>
+      <c r="K11" s="67"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12" s="63"/>
+      <c r="B12" s="64"/>
+      <c r="C12" s="64"/>
+      <c r="D12" s="64"/>
+      <c r="E12" s="64"/>
+      <c r="F12" s="64"/>
+      <c r="G12" s="66"/>
+      <c r="H12" s="66"/>
+      <c r="I12" s="66"/>
+      <c r="J12" s="66"/>
+      <c r="K12" s="67"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" s="63"/>
+      <c r="B13" s="64"/>
+      <c r="C13" s="64"/>
+      <c r="D13" s="64"/>
+      <c r="E13" s="64"/>
+      <c r="F13" s="64"/>
+      <c r="G13" s="66"/>
+      <c r="H13" s="66"/>
+      <c r="I13" s="66"/>
+      <c r="J13" s="66"/>
+      <c r="K13" s="67"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A14" s="63"/>
+      <c r="B14" s="64"/>
+      <c r="C14" s="64"/>
+      <c r="D14" s="64"/>
+      <c r="E14" s="64"/>
+      <c r="F14" s="64"/>
+      <c r="G14" s="66"/>
+      <c r="H14" s="66"/>
+      <c r="I14" s="66"/>
+      <c r="J14" s="66"/>
+      <c r="K14" s="67"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3274,46 +2816,46 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:Q11"/>
-  <sheetFormatPr defaultColWidth="11.36328125" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.08984375" style="23" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.08984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.08984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.08984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.08984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="27.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="32.08984375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="29.08984375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="24.08984375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20.08984375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="24.36328125" customWidth="1"/>
-    <col min="16" max="17" width="20.08984375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="22.08984375" customWidth="1"/>
+    <col min="1" max="1" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" style="23" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="32.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="24.42578125" customWidth="1"/>
+    <col min="16" max="17" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="22.140625" customWidth="1"/>
     <col min="19" max="19" width="22" customWidth="1"/>
-    <col min="20" max="20" width="15.7265625" customWidth="1"/>
+    <col min="20" max="20" width="15.7109375" customWidth="1"/>
     <col min="21" max="21" width="14" customWidth="1"/>
-    <col min="22" max="22" width="17.6328125" customWidth="1"/>
+    <col min="22" max="22" width="17.5703125" customWidth="1"/>
     <col min="23" max="23" width="16" customWidth="1"/>
     <col min="24" max="24" width="25" customWidth="1"/>
-    <col min="25" max="25" width="19.81640625" customWidth="1"/>
-    <col min="26" max="26" width="10.08984375" customWidth="1"/>
-    <col min="27" max="27" width="7.81640625" customWidth="1"/>
-    <col min="28" max="28" width="8.7265625" customWidth="1"/>
-    <col min="29" max="29" width="9.6328125" customWidth="1"/>
-    <col min="30" max="30" width="8.7265625" customWidth="1"/>
-    <col min="31" max="31" width="29.36328125" customWidth="1"/>
+    <col min="25" max="25" width="19.85546875" customWidth="1"/>
+    <col min="26" max="26" width="10.140625" customWidth="1"/>
+    <col min="27" max="27" width="7.85546875" customWidth="1"/>
+    <col min="28" max="28" width="8.7109375" customWidth="1"/>
+    <col min="29" max="29" width="9.5703125" customWidth="1"/>
+    <col min="30" max="30" width="8.7109375" customWidth="1"/>
+    <col min="31" max="31" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="31" t="s">
         <v>16</v>
       </c>
@@ -3321,7 +2863,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="29" t="s">
-        <v>79</v>
+        <v>44</v>
       </c>
       <c r="D3" s="30" t="s">
         <v>23</v>
@@ -3348,30 +2890,30 @@
         <v>30</v>
       </c>
       <c r="L3" s="30" t="s">
-        <v>80</v>
+        <v>45</v>
       </c>
       <c r="M3" s="30" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
       <c r="N3" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="O3" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="O3" s="13" t="s">
-        <v>117</v>
-      </c>
       <c r="P3" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q3" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="Q3" s="13" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>17</v>
       </c>
       <c r="B4" s="38" t="s">
-        <v>141</v>
+        <v>92</v>
       </c>
       <c r="C4" s="32">
         <v>5</v>
@@ -3419,12 +2961,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
       <c r="B5" s="38" t="s">
-        <v>142</v>
+        <v>93</v>
       </c>
       <c r="C5" s="32">
         <v>4</v>
@@ -3472,12 +3014,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B6" s="38" t="s">
-        <v>143</v>
+        <v>94</v>
       </c>
       <c r="C6" s="32">
         <v>3</v>
@@ -3525,12 +3067,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B7" s="38" t="s">
-        <v>144</v>
+        <v>95</v>
       </c>
       <c r="C7" s="32">
         <v>2</v>
@@ -3578,12 +3120,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:17" s="18" customFormat="1" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" s="18" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>21</v>
       </c>
       <c r="B8" s="62" t="s">
-        <v>145</v>
+        <v>96</v>
       </c>
       <c r="C8" s="33">
         <v>3</v>
@@ -3631,7 +3173,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C9" s="18"/>
       <c r="D9" s="18"/>
       <c r="E9" s="18"/>
@@ -3644,10 +3186,10 @@
       <c r="L9" s="18"/>
       <c r="M9" s="18"/>
     </row>
-    <row r="10" spans="1:17" s="18" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="24"/>
       <c r="B10" s="24" t="s">
-        <v>78</v>
+        <v>43</v>
       </c>
       <c r="C10" s="50">
         <f>AVERAGE(C4:C8)</f>
@@ -3710,7 +3252,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:17" s="18" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:17" s="18" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="24"/>
       <c r="B11" s="24" t="s">
         <v>5</v>

</xml_diff>

<commit_message>
Add one to data-ta.xlsx
</commit_message>
<xml_diff>
--- a/g1-09-ta/data-ta.xlsx
+++ b/g1-09-ta/data-ta.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Uni\HCI\hci-ex3\g1-09-ta\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sven\Documents\School\Radboud\Computing Science\Minor\Vakken\Human-Computer Interaction\Ex3\hci-ex3\g1-09-ta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2EE88A9-A081-42E5-90C7-7784388F1C5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CBDB0FF-C588-4382-902D-4F31C5D8CBA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="503" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="503" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Background Q" sheetId="3" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="152">
   <si>
     <t>Browser</t>
   </si>
@@ -476,6 +476,21 @@
   </si>
   <si>
     <t>TP1 00:02:23</t>
+  </si>
+  <si>
+    <t>n-tp2-annoying-order-by-midnight.mp4</t>
+  </si>
+  <si>
+    <t>TP2 00:20:49</t>
+  </si>
+  <si>
+    <t>The user is annoyed by the AlzaBox banner  saying order by midnight at a lot of products</t>
+  </si>
+  <si>
+    <t>Annoying Order by Midnight</t>
+  </si>
+  <si>
+    <t>Homepage → Components → PC Builder → PC Configurator → Graphics Card</t>
   </si>
 </sst>
 </file>
@@ -1106,8 +1121,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Link" xfId="1" builtinId="8"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1410,43 +1425,43 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" customWidth="1"/>
-    <col min="2" max="2" width="12.140625" customWidth="1"/>
-    <col min="3" max="3" width="11.28515625" customWidth="1"/>
-    <col min="4" max="4" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.54296875" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" customWidth="1"/>
+    <col min="3" max="3" width="11.26953125" customWidth="1"/>
+    <col min="4" max="4" width="5.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.26953125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="23" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
-    <col min="9" max="9" width="6.7109375" customWidth="1"/>
-    <col min="10" max="10" width="7.85546875" customWidth="1"/>
-    <col min="11" max="11" width="13.5703125" customWidth="1"/>
-    <col min="12" max="12" width="6.28515625" customWidth="1"/>
-    <col min="13" max="13" width="7.140625" customWidth="1"/>
-    <col min="14" max="14" width="13.5703125" customWidth="1"/>
-    <col min="15" max="15" width="6.28515625" customWidth="1"/>
-    <col min="16" max="16" width="7.5703125" customWidth="1"/>
-    <col min="17" max="17" width="13.42578125" customWidth="1"/>
-    <col min="18" max="18" width="12.7109375" customWidth="1"/>
+    <col min="9" max="9" width="6.7265625" customWidth="1"/>
+    <col min="10" max="10" width="7.81640625" customWidth="1"/>
+    <col min="11" max="11" width="13.54296875" customWidth="1"/>
+    <col min="12" max="12" width="6.26953125" customWidth="1"/>
+    <col min="13" max="13" width="7.1796875" customWidth="1"/>
+    <col min="14" max="14" width="13.54296875" customWidth="1"/>
+    <col min="15" max="15" width="6.26953125" customWidth="1"/>
+    <col min="16" max="16" width="7.54296875" customWidth="1"/>
+    <col min="17" max="17" width="13.453125" customWidth="1"/>
+    <col min="18" max="18" width="12.7265625" customWidth="1"/>
     <col min="19" max="19" width="14" customWidth="1"/>
-    <col min="20" max="20" width="8.28515625" customWidth="1"/>
-    <col min="21" max="21" width="15.28515625" customWidth="1"/>
-    <col min="22" max="22" width="13.42578125" customWidth="1"/>
-    <col min="23" max="23" width="13.5703125" customWidth="1"/>
-    <col min="24" max="24" width="13.85546875" customWidth="1"/>
-    <col min="25" max="25" width="13.140625" customWidth="1"/>
-    <col min="26" max="26" width="22.42578125" customWidth="1"/>
+    <col min="20" max="20" width="8.26953125" customWidth="1"/>
+    <col min="21" max="21" width="15.26953125" customWidth="1"/>
+    <col min="22" max="22" width="13.453125" customWidth="1"/>
+    <col min="23" max="23" width="13.54296875" customWidth="1"/>
+    <col min="24" max="24" width="13.81640625" customWidth="1"/>
+    <col min="25" max="25" width="13.1796875" customWidth="1"/>
+    <col min="26" max="26" width="22.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:26" ht="13" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="1:26" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:26" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="C3" s="9" t="s">
         <v>49</v>
       </c>
@@ -1488,7 +1503,7 @@
       <c r="Y3" s="78"/>
       <c r="Z3" s="11"/>
     </row>
-    <row r="4" spans="1:26" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:26" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="31" t="s">
         <v>16</v>
       </c>
@@ -1568,7 +1583,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>17</v>
       </c>
@@ -1648,7 +1663,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
@@ -1728,7 +1743,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
@@ -1808,7 +1823,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -1888,7 +1903,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
         <v>21</v>
       </c>
@@ -1968,7 +1983,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="10" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I10" s="18"/>
       <c r="J10" s="18"/>
       <c r="L10" s="18"/>
@@ -1976,7 +1991,7 @@
       <c r="O10" s="18"/>
       <c r="P10" s="18"/>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:26" ht="13" x14ac:dyDescent="0.3">
       <c r="A11" s="24"/>
       <c r="B11" s="26" t="s">
         <v>43</v>
@@ -2032,7 +2047,7 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="24"/>
       <c r="B12" s="26" t="s">
         <v>14</v>
@@ -2083,7 +2098,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
       <c r="H13" t="s">
         <v>62</v>
       </c>
@@ -2110,22 +2125,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.140625" style="23" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" customWidth="1"/>
-    <col min="5" max="5" width="11.7109375" customWidth="1"/>
-    <col min="6" max="7" width="10.7109375" customWidth="1"/>
+    <col min="1" max="1" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" style="23" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.7265625" customWidth="1"/>
+    <col min="4" max="4" width="15.7265625" customWidth="1"/>
+    <col min="5" max="5" width="11.7265625" customWidth="1"/>
+    <col min="6" max="7" width="10.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="13" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" ht="13" x14ac:dyDescent="0.3">
       <c r="C3" s="35" t="s">
         <v>4</v>
       </c>
@@ -2134,7 +2149,7 @@
       <c r="F3" s="25"/>
       <c r="G3" s="25"/>
     </row>
-    <row r="4" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="31" t="s">
         <v>16</v>
       </c>
@@ -2157,7 +2172,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>17</v>
       </c>
@@ -2180,7 +2195,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
@@ -2203,7 +2218,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
@@ -2226,7 +2241,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -2249,7 +2264,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="19" t="s">
         <v>21</v>
       </c>
@@ -2272,7 +2287,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="24"/>
       <c r="B10" s="24" t="s">
         <v>2</v>
@@ -2298,7 +2313,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" ht="13" x14ac:dyDescent="0.3">
       <c r="A11" s="24"/>
       <c r="B11" s="24" t="s">
         <v>3</v>
@@ -2335,29 +2350,29 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
-    <col min="2" max="2" width="36.140625" customWidth="1"/>
-    <col min="3" max="3" width="35.140625" customWidth="1"/>
-    <col min="4" max="4" width="34.42578125" customWidth="1"/>
-    <col min="5" max="5" width="25.85546875" customWidth="1"/>
+    <col min="2" max="2" width="36.1796875" customWidth="1"/>
+    <col min="3" max="3" width="35.1796875" customWidth="1"/>
+    <col min="4" max="4" width="34.453125" customWidth="1"/>
+    <col min="5" max="5" width="25.81640625" customWidth="1"/>
     <col min="6" max="6" width="29" customWidth="1"/>
-    <col min="7" max="10" width="4.5703125" style="55" customWidth="1"/>
-    <col min="11" max="11" width="6.140625" style="55" customWidth="1"/>
+    <col min="7" max="10" width="4.54296875" style="55" customWidth="1"/>
+    <col min="11" max="11" width="6.1796875" style="55" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" ht="13" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" ht="13" x14ac:dyDescent="0.3">
       <c r="G3" s="58" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:11" s="56" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" s="56" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="60" t="s">
         <v>32</v>
       </c>
@@ -2392,7 +2407,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A5" s="63">
         <v>1</v>
       </c>
@@ -2420,7 +2435,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A6" s="63">
         <v>2</v>
       </c>
@@ -2448,7 +2463,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A7" s="63">
         <v>3</v>
       </c>
@@ -2476,7 +2491,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A8" s="63">
         <v>4</v>
       </c>
@@ -2504,20 +2519,37 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" s="63"/>
-      <c r="B9" s="64"/>
-      <c r="C9" s="64"/>
-      <c r="D9" s="63"/>
-      <c r="E9" s="63"/>
-      <c r="F9" s="69"/>
+    <row r="9" spans="1:11" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="63">
+        <v>5</v>
+      </c>
+      <c r="B9" s="64" t="s">
+        <v>150</v>
+      </c>
+      <c r="C9" s="64" t="s">
+        <v>149</v>
+      </c>
+      <c r="D9" s="63" t="s">
+        <v>147</v>
+      </c>
+      <c r="E9" s="63" t="s">
+        <v>148</v>
+      </c>
+      <c r="F9" s="69" t="s">
+        <v>151</v>
+      </c>
       <c r="G9" s="66"/>
       <c r="H9" s="66"/>
       <c r="I9" s="66"/>
-      <c r="J9" s="66"/>
-      <c r="K9" s="67"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J9" s="66">
+        <v>1</v>
+      </c>
+      <c r="K9" s="67">
+        <f>AVERAGE(G9:J9)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="63"/>
       <c r="B10" s="64"/>
       <c r="C10" s="64"/>
@@ -2530,7 +2562,7 @@
       <c r="J10" s="66"/>
       <c r="K10" s="67"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="63"/>
       <c r="B11" s="64"/>
       <c r="C11" s="64"/>
@@ -2543,7 +2575,7 @@
       <c r="J11" s="66"/>
       <c r="K11" s="67"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="68"/>
       <c r="B12" s="69"/>
       <c r="C12" s="69"/>
@@ -2556,7 +2588,7 @@
       <c r="J12" s="66"/>
       <c r="K12" s="67"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="68"/>
       <c r="B13" s="69"/>
       <c r="C13" s="69"/>
@@ -2569,7 +2601,7 @@
       <c r="J13" s="66"/>
       <c r="K13" s="67"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="63"/>
       <c r="B14" s="64"/>
       <c r="C14" s="64"/>
@@ -2591,28 +2623,28 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
-    <col min="3" max="4" width="35.140625" customWidth="1"/>
-    <col min="5" max="5" width="26.140625" customWidth="1"/>
-    <col min="6" max="6" width="29.140625" customWidth="1"/>
-    <col min="7" max="10" width="4.5703125" style="55" customWidth="1"/>
-    <col min="11" max="11" width="5.85546875" style="55" customWidth="1"/>
+    <col min="3" max="4" width="35.1796875" customWidth="1"/>
+    <col min="5" max="5" width="26.1796875" customWidth="1"/>
+    <col min="6" max="6" width="29.1796875" customWidth="1"/>
+    <col min="7" max="10" width="4.54296875" style="55" customWidth="1"/>
+    <col min="11" max="11" width="5.81640625" style="55" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" ht="13" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" ht="13" x14ac:dyDescent="0.3">
       <c r="G3" s="58" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:11" s="56" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" s="56" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="60" t="s">
         <v>32</v>
       </c>
@@ -2647,7 +2679,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" ht="25" x14ac:dyDescent="0.25">
       <c r="A5" s="63">
         <v>1</v>
       </c>
@@ -2675,7 +2707,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" ht="25" x14ac:dyDescent="0.25">
       <c r="A6" s="63">
         <v>2</v>
       </c>
@@ -2703,7 +2735,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="63"/>
       <c r="B7" s="64"/>
       <c r="C7" s="64"/>
@@ -2716,7 +2748,7 @@
       <c r="J7" s="66"/>
       <c r="K7" s="67"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="63"/>
       <c r="B8" s="64"/>
       <c r="C8" s="64"/>
@@ -2729,7 +2761,7 @@
       <c r="J8" s="66"/>
       <c r="K8" s="67"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="63"/>
       <c r="B9" s="64"/>
       <c r="C9" s="64"/>
@@ -2742,7 +2774,7 @@
       <c r="J9" s="66"/>
       <c r="K9" s="67"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="63"/>
       <c r="B10" s="64"/>
       <c r="C10" s="64"/>
@@ -2755,7 +2787,7 @@
       <c r="J10" s="66"/>
       <c r="K10" s="67"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="63"/>
       <c r="B11" s="64"/>
       <c r="C11" s="64"/>
@@ -2768,7 +2800,7 @@
       <c r="J11" s="66"/>
       <c r="K11" s="67"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="63"/>
       <c r="B12" s="64"/>
       <c r="C12" s="64"/>
@@ -2781,7 +2813,7 @@
       <c r="J12" s="66"/>
       <c r="K12" s="67"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="63"/>
       <c r="B13" s="64"/>
       <c r="C13" s="64"/>
@@ -2794,7 +2826,7 @@
       <c r="J13" s="66"/>
       <c r="K13" s="67"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="63"/>
       <c r="B14" s="64"/>
       <c r="C14" s="64"/>
@@ -2816,46 +2848,46 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:Q11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.140625" style="23" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="27.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="32.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="29.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="24.42578125" customWidth="1"/>
-    <col min="16" max="17" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="22.140625" customWidth="1"/>
+    <col min="1" max="1" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" style="23" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="32.1796875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="29.1796875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24.1796875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.1796875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="24.453125" customWidth="1"/>
+    <col min="16" max="17" width="20.1796875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="22.1796875" customWidth="1"/>
     <col min="19" max="19" width="22" customWidth="1"/>
-    <col min="20" max="20" width="15.7109375" customWidth="1"/>
+    <col min="20" max="20" width="15.7265625" customWidth="1"/>
     <col min="21" max="21" width="14" customWidth="1"/>
-    <col min="22" max="22" width="17.5703125" customWidth="1"/>
+    <col min="22" max="22" width="17.54296875" customWidth="1"/>
     <col min="23" max="23" width="16" customWidth="1"/>
     <col min="24" max="24" width="25" customWidth="1"/>
-    <col min="25" max="25" width="19.85546875" customWidth="1"/>
-    <col min="26" max="26" width="10.140625" customWidth="1"/>
-    <col min="27" max="27" width="7.85546875" customWidth="1"/>
-    <col min="28" max="28" width="8.7109375" customWidth="1"/>
-    <col min="29" max="29" width="9.5703125" customWidth="1"/>
-    <col min="30" max="30" width="8.7109375" customWidth="1"/>
-    <col min="31" max="31" width="29.42578125" customWidth="1"/>
+    <col min="25" max="25" width="19.81640625" customWidth="1"/>
+    <col min="26" max="26" width="10.1796875" customWidth="1"/>
+    <col min="27" max="27" width="7.81640625" customWidth="1"/>
+    <col min="28" max="28" width="8.7265625" customWidth="1"/>
+    <col min="29" max="29" width="9.54296875" customWidth="1"/>
+    <col min="30" max="30" width="8.7265625" customWidth="1"/>
+    <col min="31" max="31" width="29.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:17" ht="13" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="3" spans="1:17" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="31" t="s">
         <v>16</v>
       </c>
@@ -2908,7 +2940,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="4" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>17</v>
       </c>
@@ -2961,7 +2993,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
@@ -3014,7 +3046,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>19</v>
       </c>
@@ -3067,7 +3099,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -3120,7 +3152,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:17" s="18" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" s="18" customFormat="1" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="19" t="s">
         <v>21</v>
       </c>
@@ -3173,7 +3205,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C9" s="18"/>
       <c r="D9" s="18"/>
       <c r="E9" s="18"/>
@@ -3186,7 +3218,7 @@
       <c r="L9" s="18"/>
       <c r="M9" s="18"/>
     </row>
-    <row r="10" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:17" s="18" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A10" s="24"/>
       <c r="B10" s="24" t="s">
         <v>43</v>
@@ -3252,7 +3284,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:17" s="18" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" s="18" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="24"/>
       <c r="B11" s="24" t="s">
         <v>5</v>

</xml_diff>

<commit_message>
Removed 1 Positive Finding, added clip names to excel, created clips for tp1 findings
</commit_message>
<xml_diff>
--- a/g1-09-ta/data-ta.xlsx
+++ b/g1-09-ta/data-ta.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sven\Documents\School\Radboud\Computing Science\Minor\Vakken\Human-Computer Interaction\Ex3\hci-ex3\g1-09-ta\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Uni\HCI\hci-ex3\g1-09-ta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BE2F205-2A23-4664-821A-B680F06215B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{136EE6E1-0252-4F7C-806A-EA57D591A2C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="503" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="503" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Background Q" sheetId="3" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="225">
   <si>
     <t>Browser</t>
   </si>
@@ -457,12 +457,6 @@
     <t>TP1 00:11:28</t>
   </si>
   <si>
-    <t>The user is able to quickly change the website language without any difficulties</t>
-  </si>
-  <si>
-    <t>TP1 00:00:30</t>
-  </si>
-  <si>
     <t>Homepage</t>
   </si>
   <si>
@@ -472,9 +466,6 @@
     <t>Easy Navigation for New Users</t>
   </si>
   <si>
-    <t>Simple Language Switch</t>
-  </si>
-  <si>
     <t>TP1 00:02:23</t>
   </si>
   <si>
@@ -499,9 +490,6 @@
     <t>Missing Apple Subcategory</t>
   </si>
   <si>
-    <t>n-tp1-x-x-x-x.mp4, n-tp2-random-another-language.mp4</t>
-  </si>
-  <si>
     <t>n-tp2-little-filtering.mp4</t>
   </si>
   <si>
@@ -707,6 +695,21 @@
   </si>
   <si>
     <t>Checkout → payment step, first checkout after registration (it should take information eg. adres from registration form, bcs we inserted it there)</t>
+  </si>
+  <si>
+    <t>n-tp1-wrong-language.mp4, n-tp2-random-another-language.mp4</t>
+  </si>
+  <si>
+    <t>p-tp1-easy-to-use.mp4</t>
+  </si>
+  <si>
+    <t>n-tp1-similar-products.mp4</t>
+  </si>
+  <si>
+    <t>n-tp1-overlapping-bug.mp4</t>
+  </si>
+  <si>
+    <t>n-tp1-unclear-green-details.mp4</t>
   </si>
 </sst>
 </file>
@@ -1324,7 +1327,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1627,43 +1630,43 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z13"/>
-  <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.54296875" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" customWidth="1"/>
-    <col min="3" max="3" width="11.26953125" customWidth="1"/>
-    <col min="4" max="4" width="5.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" customWidth="1"/>
+    <col min="3" max="3" width="11.28515625" customWidth="1"/>
+    <col min="4" max="4" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="23" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
-    <col min="9" max="9" width="6.7265625" customWidth="1"/>
-    <col min="10" max="10" width="7.81640625" customWidth="1"/>
-    <col min="11" max="11" width="13.54296875" customWidth="1"/>
-    <col min="12" max="12" width="6.26953125" customWidth="1"/>
-    <col min="13" max="13" width="7.1796875" customWidth="1"/>
-    <col min="14" max="14" width="13.54296875" customWidth="1"/>
-    <col min="15" max="15" width="6.26953125" customWidth="1"/>
-    <col min="16" max="16" width="7.54296875" customWidth="1"/>
-    <col min="17" max="17" width="13.453125" customWidth="1"/>
-    <col min="18" max="18" width="12.7265625" customWidth="1"/>
+    <col min="9" max="9" width="6.7109375" customWidth="1"/>
+    <col min="10" max="10" width="7.85546875" customWidth="1"/>
+    <col min="11" max="11" width="13.5703125" customWidth="1"/>
+    <col min="12" max="12" width="6.28515625" customWidth="1"/>
+    <col min="13" max="13" width="7.140625" customWidth="1"/>
+    <col min="14" max="14" width="13.5703125" customWidth="1"/>
+    <col min="15" max="15" width="6.28515625" customWidth="1"/>
+    <col min="16" max="16" width="7.5703125" customWidth="1"/>
+    <col min="17" max="17" width="13.42578125" customWidth="1"/>
+    <col min="18" max="18" width="12.7109375" customWidth="1"/>
     <col min="19" max="19" width="14" customWidth="1"/>
-    <col min="20" max="20" width="8.26953125" customWidth="1"/>
-    <col min="21" max="21" width="15.26953125" customWidth="1"/>
-    <col min="22" max="22" width="13.453125" customWidth="1"/>
-    <col min="23" max="23" width="13.54296875" customWidth="1"/>
-    <col min="24" max="24" width="13.81640625" customWidth="1"/>
-    <col min="25" max="25" width="13.1796875" customWidth="1"/>
-    <col min="26" max="26" width="22.453125" customWidth="1"/>
+    <col min="20" max="20" width="8.28515625" customWidth="1"/>
+    <col min="21" max="21" width="15.28515625" customWidth="1"/>
+    <col min="22" max="22" width="13.42578125" customWidth="1"/>
+    <col min="23" max="23" width="13.5703125" customWidth="1"/>
+    <col min="24" max="24" width="13.85546875" customWidth="1"/>
+    <col min="25" max="25" width="13.140625" customWidth="1"/>
+    <col min="26" max="26" width="22.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:26" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:26" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C3" s="9" t="s">
         <v>49</v>
       </c>
@@ -1705,7 +1708,7 @@
       <c r="Y3" s="77"/>
       <c r="Z3" s="11"/>
     </row>
-    <row r="4" spans="1:26" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:26" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="31" t="s">
         <v>16</v>
       </c>
@@ -1785,7 +1788,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>17</v>
       </c>
@@ -1865,7 +1868,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
@@ -1945,7 +1948,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
@@ -2025,7 +2028,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -2105,7 +2108,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A9" s="19" t="s">
         <v>21</v>
       </c>
@@ -2185,7 +2188,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="10" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="I10" s="18"/>
       <c r="J10" s="18"/>
       <c r="L10" s="18"/>
@@ -2193,7 +2196,7 @@
       <c r="O10" s="18"/>
       <c r="P10" s="18"/>
     </row>
-    <row r="11" spans="1:26" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A11" s="24"/>
       <c r="B11" s="26" t="s">
         <v>43</v>
@@ -2249,7 +2252,7 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="24"/>
       <c r="B12" s="26" t="s">
         <v>14</v>
@@ -2300,7 +2303,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.2">
       <c r="H13" t="s">
         <v>62</v>
       </c>
@@ -2327,22 +2330,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" style="23" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7265625" customWidth="1"/>
-    <col min="4" max="4" width="15.7265625" customWidth="1"/>
-    <col min="5" max="5" width="11.7265625" customWidth="1"/>
-    <col min="6" max="7" width="10.7265625" customWidth="1"/>
+    <col min="1" max="1" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" style="23" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" customWidth="1"/>
+    <col min="6" max="7" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C3" s="35" t="s">
         <v>4</v>
       </c>
@@ -2351,7 +2354,7 @@
       <c r="F3" s="25"/>
       <c r="G3" s="25"/>
     </row>
-    <row r="4" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="31" t="s">
         <v>16</v>
       </c>
@@ -2374,7 +2377,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>17</v>
       </c>
@@ -2397,7 +2400,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
@@ -2420,7 +2423,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
@@ -2443,7 +2446,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -2466,7 +2469,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
         <v>21</v>
       </c>
@@ -2489,7 +2492,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="24"/>
       <c r="B10" s="24" t="s">
         <v>2</v>
@@ -2515,7 +2518,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="24"/>
       <c r="B11" s="24" t="s">
         <v>3</v>
@@ -2552,29 +2555,29 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K19"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
-    <col min="2" max="2" width="36.1796875" customWidth="1"/>
-    <col min="3" max="3" width="35.1796875" customWidth="1"/>
-    <col min="4" max="4" width="34.453125" customWidth="1"/>
-    <col min="5" max="5" width="25.81640625" customWidth="1"/>
+    <col min="2" max="2" width="36.140625" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" customWidth="1"/>
+    <col min="4" max="4" width="34.42578125" customWidth="1"/>
+    <col min="5" max="5" width="25.85546875" customWidth="1"/>
     <col min="6" max="6" width="29" customWidth="1"/>
-    <col min="7" max="10" width="4.54296875" style="55" customWidth="1"/>
-    <col min="11" max="11" width="6.1796875" style="55" customWidth="1"/>
+    <col min="7" max="10" width="4.5703125" style="55" customWidth="1"/>
+    <col min="11" max="11" width="6.140625" style="55" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="G3" s="58" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:11" s="56" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" s="56" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="60" t="s">
         <v>32</v>
       </c>
@@ -2609,7 +2612,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A5" s="63">
         <v>1</v>
       </c>
@@ -2620,7 +2623,7 @@
         <v>121</v>
       </c>
       <c r="D5" s="69" t="s">
-        <v>154</v>
+        <v>220</v>
       </c>
       <c r="E5" s="69" t="s">
         <v>123</v>
@@ -2641,7 +2644,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A6" s="63">
         <v>2</v>
       </c>
@@ -2651,7 +2654,9 @@
       <c r="C6" s="64" t="s">
         <v>129</v>
       </c>
-      <c r="D6" s="63"/>
+      <c r="D6" s="63" t="s">
+        <v>222</v>
+      </c>
       <c r="E6" s="63" t="s">
         <v>131</v>
       </c>
@@ -2669,7 +2674,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A7" s="63">
         <v>3</v>
       </c>
@@ -2679,7 +2684,9 @@
       <c r="C7" s="64" t="s">
         <v>134</v>
       </c>
-      <c r="D7" s="63"/>
+      <c r="D7" s="63" t="s">
+        <v>223</v>
+      </c>
       <c r="E7" s="63" t="s">
         <v>135</v>
       </c>
@@ -2697,7 +2704,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A8" s="63">
         <v>4</v>
       </c>
@@ -2707,7 +2714,9 @@
       <c r="C8" s="64" t="s">
         <v>137</v>
       </c>
-      <c r="D8" s="63"/>
+      <c r="D8" s="63" t="s">
+        <v>224</v>
+      </c>
       <c r="E8" s="69" t="s">
         <v>139</v>
       </c>
@@ -2725,24 +2734,24 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A9" s="63">
         <v>5</v>
       </c>
       <c r="B9" s="64" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C9" s="64" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D9" s="63" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="E9" s="63" t="s">
+        <v>145</v>
+      </c>
+      <c r="F9" s="69" t="s">
         <v>148</v>
-      </c>
-      <c r="F9" s="69" t="s">
-        <v>151</v>
       </c>
       <c r="G9" s="66">
         <v>1</v>
@@ -2759,24 +2768,24 @@
         <v>1.3333333333333333</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A10" s="63">
         <v>6</v>
       </c>
       <c r="B10" s="64" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C10" s="64" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="D10" s="63" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="E10" s="63" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="F10" s="69" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="G10" s="66">
         <v>2</v>
@@ -2789,24 +2798,24 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A11" s="63">
         <v>7</v>
       </c>
       <c r="B11" s="64" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C11" s="64" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="D11" s="63" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="E11" s="63" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="F11" s="64" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="G11" s="66">
         <v>2</v>
@@ -2819,24 +2828,24 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A12" s="68" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B12" s="69" t="s">
+        <v>180</v>
+      </c>
+      <c r="C12" s="69" t="s">
+        <v>181</v>
+      </c>
+      <c r="D12" s="65" t="s">
+        <v>182</v>
+      </c>
+      <c r="E12" s="65" t="s">
+        <v>183</v>
+      </c>
+      <c r="F12" s="69" t="s">
         <v>184</v>
-      </c>
-      <c r="C12" s="69" t="s">
-        <v>185</v>
-      </c>
-      <c r="D12" s="65" t="s">
-        <v>186</v>
-      </c>
-      <c r="E12" s="65" t="s">
-        <v>187</v>
-      </c>
-      <c r="F12" s="69" t="s">
-        <v>188</v>
       </c>
       <c r="G12" s="66"/>
       <c r="H12" s="66"/>
@@ -2849,24 +2858,24 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="50" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A13" s="68" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B13" s="69" t="s">
+        <v>185</v>
+      </c>
+      <c r="C13" s="69" t="s">
+        <v>186</v>
+      </c>
+      <c r="D13" s="65" t="s">
+        <v>187</v>
+      </c>
+      <c r="E13" s="65" t="s">
+        <v>188</v>
+      </c>
+      <c r="F13" s="69" t="s">
         <v>189</v>
-      </c>
-      <c r="C13" s="69" t="s">
-        <v>190</v>
-      </c>
-      <c r="D13" s="65" t="s">
-        <v>191</v>
-      </c>
-      <c r="E13" s="65" t="s">
-        <v>192</v>
-      </c>
-      <c r="F13" s="69" t="s">
-        <v>193</v>
       </c>
       <c r="G13" s="66"/>
       <c r="H13" s="66"/>
@@ -2879,24 +2888,24 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="50" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A14" s="68" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B14" s="69" t="s">
+        <v>190</v>
+      </c>
+      <c r="C14" s="69" t="s">
+        <v>191</v>
+      </c>
+      <c r="D14" s="65" t="s">
+        <v>192</v>
+      </c>
+      <c r="E14" s="65" t="s">
+        <v>193</v>
+      </c>
+      <c r="F14" s="69" t="s">
         <v>194</v>
-      </c>
-      <c r="C14" s="69" t="s">
-        <v>195</v>
-      </c>
-      <c r="D14" s="65" t="s">
-        <v>196</v>
-      </c>
-      <c r="E14" s="65" t="s">
-        <v>197</v>
-      </c>
-      <c r="F14" s="69" t="s">
-        <v>198</v>
       </c>
       <c r="G14" s="66"/>
       <c r="H14" s="66"/>
@@ -2909,24 +2918,24 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="50" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A15" s="68" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B15" s="69" t="s">
+        <v>195</v>
+      </c>
+      <c r="C15" s="69" t="s">
+        <v>196</v>
+      </c>
+      <c r="D15" s="65" t="s">
+        <v>197</v>
+      </c>
+      <c r="E15" s="65" t="s">
+        <v>198</v>
+      </c>
+      <c r="F15" s="69" t="s">
         <v>199</v>
-      </c>
-      <c r="C15" s="69" t="s">
-        <v>200</v>
-      </c>
-      <c r="D15" s="65" t="s">
-        <v>201</v>
-      </c>
-      <c r="E15" s="65" t="s">
-        <v>202</v>
-      </c>
-      <c r="F15" s="69" t="s">
-        <v>203</v>
       </c>
       <c r="G15" s="66"/>
       <c r="H15" s="66"/>
@@ -2939,24 +2948,24 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A16" s="68" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B16" s="69" t="s">
+        <v>200</v>
+      </c>
+      <c r="C16" s="69" t="s">
+        <v>201</v>
+      </c>
+      <c r="D16" s="65" t="s">
+        <v>202</v>
+      </c>
+      <c r="E16" s="65" t="s">
+        <v>203</v>
+      </c>
+      <c r="F16" s="69" t="s">
         <v>204</v>
-      </c>
-      <c r="C16" s="69" t="s">
-        <v>205</v>
-      </c>
-      <c r="D16" s="65" t="s">
-        <v>206</v>
-      </c>
-      <c r="E16" s="65" t="s">
-        <v>207</v>
-      </c>
-      <c r="F16" s="69" t="s">
-        <v>208</v>
       </c>
       <c r="G16" s="66"/>
       <c r="H16" s="66"/>
@@ -2969,24 +2978,24 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="50" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A17" s="68" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B17" s="69" t="s">
+        <v>205</v>
+      </c>
+      <c r="C17" s="69" t="s">
+        <v>206</v>
+      </c>
+      <c r="D17" s="65" t="s">
+        <v>207</v>
+      </c>
+      <c r="E17" s="65" t="s">
+        <v>208</v>
+      </c>
+      <c r="F17" s="69" t="s">
         <v>209</v>
-      </c>
-      <c r="C17" s="69" t="s">
-        <v>210</v>
-      </c>
-      <c r="D17" s="65" t="s">
-        <v>211</v>
-      </c>
-      <c r="E17" s="65" t="s">
-        <v>212</v>
-      </c>
-      <c r="F17" s="69" t="s">
-        <v>213</v>
       </c>
       <c r="G17" s="66"/>
       <c r="H17" s="66"/>
@@ -2999,24 +3008,24 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="50" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A18" s="68" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B18" s="69" t="s">
+        <v>210</v>
+      </c>
+      <c r="C18" s="69" t="s">
+        <v>211</v>
+      </c>
+      <c r="D18" s="65" t="s">
+        <v>212</v>
+      </c>
+      <c r="E18" s="65" t="s">
+        <v>213</v>
+      </c>
+      <c r="F18" s="69" t="s">
         <v>214</v>
-      </c>
-      <c r="C18" s="69" t="s">
-        <v>215</v>
-      </c>
-      <c r="D18" s="65" t="s">
-        <v>216</v>
-      </c>
-      <c r="E18" s="65" t="s">
-        <v>217</v>
-      </c>
-      <c r="F18" s="69" t="s">
-        <v>218</v>
       </c>
       <c r="G18" s="66"/>
       <c r="H18" s="66"/>
@@ -3029,24 +3038,24 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A19" s="68" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B19" s="69" t="s">
+        <v>215</v>
+      </c>
+      <c r="C19" s="69" t="s">
+        <v>216</v>
+      </c>
+      <c r="D19" s="65" t="s">
+        <v>217</v>
+      </c>
+      <c r="E19" s="65" t="s">
+        <v>218</v>
+      </c>
+      <c r="F19" s="69" t="s">
         <v>219</v>
-      </c>
-      <c r="C19" s="69" t="s">
-        <v>220</v>
-      </c>
-      <c r="D19" s="65" t="s">
-        <v>221</v>
-      </c>
-      <c r="E19" s="65" t="s">
-        <v>222</v>
-      </c>
-      <c r="F19" s="69" t="s">
-        <v>223</v>
       </c>
       <c r="G19" s="66"/>
       <c r="H19" s="66"/>
@@ -3068,28 +3077,28 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K14"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
-    <col min="3" max="4" width="35.1796875" customWidth="1"/>
-    <col min="5" max="5" width="26.1796875" customWidth="1"/>
-    <col min="6" max="6" width="29.1796875" customWidth="1"/>
-    <col min="7" max="10" width="4.54296875" style="55" customWidth="1"/>
-    <col min="11" max="11" width="5.81640625" style="55" customWidth="1"/>
+    <col min="3" max="4" width="35.140625" customWidth="1"/>
+    <col min="5" max="5" width="26.140625" customWidth="1"/>
+    <col min="6" max="6" width="29.140625" customWidth="1"/>
+    <col min="7" max="10" width="4.5703125" style="55" customWidth="1"/>
+    <col min="11" max="11" width="5.85546875" style="55" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="G3" s="58" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:11" s="56" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" s="56" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="60" t="s">
         <v>32</v>
       </c>
@@ -3124,110 +3133,114 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A5" s="63">
         <v>1</v>
       </c>
       <c r="B5" s="64" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C5" s="64" t="s">
+        <v>141</v>
+      </c>
+      <c r="D5" s="64" t="s">
+        <v>221</v>
+      </c>
+      <c r="E5" s="64" t="s">
+        <v>143</v>
+      </c>
+      <c r="F5" s="69" t="s">
         <v>140</v>
-      </c>
-      <c r="D5" s="69"/>
-      <c r="E5" s="69" t="s">
-        <v>141</v>
-      </c>
-      <c r="F5" s="69" t="s">
-        <v>142</v>
       </c>
       <c r="G5" s="66"/>
       <c r="H5" s="66"/>
       <c r="I5" s="66"/>
       <c r="J5" s="66">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K5" s="67">
-        <f t="shared" ref="K5:K10" si="0">AVERAGE(G5:J5)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="25" x14ac:dyDescent="0.25">
+        <f t="shared" ref="K5:K9" si="0">AVERAGE(G5:J5)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A6" s="63">
         <v>2</v>
       </c>
       <c r="B6" s="64" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
       <c r="C6" s="64" t="s">
-        <v>143</v>
-      </c>
-      <c r="D6" s="64"/>
+        <v>162</v>
+      </c>
+      <c r="D6" s="64" t="s">
+        <v>155</v>
+      </c>
       <c r="E6" s="64" t="s">
-        <v>146</v>
-      </c>
-      <c r="F6" s="69" t="s">
-        <v>142</v>
-      </c>
-      <c r="G6" s="66"/>
+        <v>156</v>
+      </c>
+      <c r="F6" s="64" t="s">
+        <v>163</v>
+      </c>
+      <c r="G6" s="66">
+        <v>2</v>
+      </c>
       <c r="H6" s="66"/>
       <c r="I6" s="66"/>
-      <c r="J6" s="66">
-        <v>2</v>
-      </c>
+      <c r="J6" s="66"/>
       <c r="K6" s="67">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="25" x14ac:dyDescent="0.25">
-      <c r="A7" s="63">
-        <v>3</v>
+    <row r="7" spans="1:11" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A7" s="63" t="s">
+        <v>164</v>
       </c>
       <c r="B7" s="64" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="C7" s="64" t="s">
         <v>166</v>
       </c>
       <c r="D7" s="64" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="E7" s="64" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="F7" s="64" t="s">
-        <v>167</v>
-      </c>
-      <c r="G7" s="66">
-        <v>2</v>
-      </c>
+        <v>169</v>
+      </c>
+      <c r="G7" s="66"/>
       <c r="H7" s="66"/>
-      <c r="I7" s="66"/>
+      <c r="I7" s="66">
+        <v>3</v>
+      </c>
       <c r="J7" s="66"/>
       <c r="K7" s="67">
         <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A8" s="63" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B8" s="64" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C8" s="64" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D8" s="64" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E8" s="64" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F8" s="64" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="G8" s="66"/>
       <c r="H8" s="66"/>
@@ -3240,67 +3253,50 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="50" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A9" s="63" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B9" s="64" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C9" s="64" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D9" s="64" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E9" s="64" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F9" s="64" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G9" s="66"/>
       <c r="H9" s="66"/>
       <c r="I9" s="66">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J9" s="66"/>
       <c r="K9" s="67">
         <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="25" x14ac:dyDescent="0.25">
-      <c r="A10" s="63" t="s">
-        <v>168</v>
-      </c>
-      <c r="B10" s="64" t="s">
-        <v>179</v>
-      </c>
-      <c r="C10" s="64" t="s">
-        <v>180</v>
-      </c>
-      <c r="D10" s="64" t="s">
-        <v>181</v>
-      </c>
-      <c r="E10" s="64" t="s">
-        <v>182</v>
-      </c>
-      <c r="F10" s="64" t="s">
-        <v>183</v>
-      </c>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" s="63"/>
+      <c r="B10" s="64"/>
+      <c r="C10" s="64"/>
+      <c r="D10" s="64"/>
+      <c r="E10" s="64"/>
+      <c r="F10" s="64"/>
       <c r="G10" s="66"/>
       <c r="H10" s="66"/>
-      <c r="I10" s="66">
-        <v>1</v>
-      </c>
+      <c r="I10" s="66"/>
       <c r="J10" s="66"/>
-      <c r="K10" s="67">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K10" s="67"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" s="63"/>
       <c r="B11" s="64"/>
       <c r="C11" s="64"/>
@@ -3313,7 +3309,7 @@
       <c r="J11" s="66"/>
       <c r="K11" s="67"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="63"/>
       <c r="B12" s="64"/>
       <c r="C12" s="64"/>
@@ -3326,7 +3322,7 @@
       <c r="J12" s="66"/>
       <c r="K12" s="67"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="63"/>
       <c r="B13" s="64"/>
       <c r="C13" s="64"/>
@@ -3339,7 +3335,7 @@
       <c r="J13" s="66"/>
       <c r="K13" s="67"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" s="63"/>
       <c r="B14" s="64"/>
       <c r="C14" s="64"/>
@@ -3361,46 +3357,46 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:Q11"/>
-  <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" style="23" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="27.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="32.1796875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="29.1796875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="24.1796875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20.1796875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="24.453125" customWidth="1"/>
-    <col min="16" max="17" width="20.1796875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="22.1796875" customWidth="1"/>
+    <col min="1" max="1" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" style="23" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="32.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="24.42578125" customWidth="1"/>
+    <col min="16" max="17" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="22.140625" customWidth="1"/>
     <col min="19" max="19" width="22" customWidth="1"/>
-    <col min="20" max="20" width="15.7265625" customWidth="1"/>
+    <col min="20" max="20" width="15.7109375" customWidth="1"/>
     <col min="21" max="21" width="14" customWidth="1"/>
-    <col min="22" max="22" width="17.54296875" customWidth="1"/>
+    <col min="22" max="22" width="17.5703125" customWidth="1"/>
     <col min="23" max="23" width="16" customWidth="1"/>
     <col min="24" max="24" width="25" customWidth="1"/>
-    <col min="25" max="25" width="19.81640625" customWidth="1"/>
-    <col min="26" max="26" width="10.1796875" customWidth="1"/>
-    <col min="27" max="27" width="7.81640625" customWidth="1"/>
-    <col min="28" max="28" width="8.7265625" customWidth="1"/>
-    <col min="29" max="29" width="9.54296875" customWidth="1"/>
-    <col min="30" max="30" width="8.7265625" customWidth="1"/>
-    <col min="31" max="31" width="29.453125" customWidth="1"/>
+    <col min="25" max="25" width="19.85546875" customWidth="1"/>
+    <col min="26" max="26" width="10.140625" customWidth="1"/>
+    <col min="27" max="27" width="7.85546875" customWidth="1"/>
+    <col min="28" max="28" width="8.7109375" customWidth="1"/>
+    <col min="29" max="29" width="9.5703125" customWidth="1"/>
+    <col min="30" max="30" width="8.7109375" customWidth="1"/>
+    <col min="31" max="31" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="3" spans="1:17" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:17" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="31" t="s">
         <v>16</v>
       </c>
@@ -3453,7 +3449,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="4" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>17</v>
       </c>
@@ -3506,7 +3502,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
@@ -3559,7 +3555,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>19</v>
       </c>
@@ -3612,7 +3608,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -3665,7 +3661,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:17" s="18" customFormat="1" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" s="18" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>21</v>
       </c>
@@ -3718,7 +3714,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C9" s="18"/>
       <c r="D9" s="18"/>
       <c r="E9" s="18"/>
@@ -3731,7 +3727,7 @@
       <c r="L9" s="18"/>
       <c r="M9" s="18"/>
     </row>
-    <row r="10" spans="1:17" s="18" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="24"/>
       <c r="B10" s="24" t="s">
         <v>43</v>
@@ -3797,7 +3793,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:17" s="18" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:17" s="18" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="24"/>
       <c r="B11" s="24" t="s">
         <v>5</v>

</xml_diff>

<commit_message>
Luca rated each finding
</commit_message>
<xml_diff>
--- a/g1-09-ta/data-ta.xlsx
+++ b/g1-09-ta/data-ta.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sven\Documents\School\Radboud\Computing Science\Minor\Vakken\Human-Computer Interaction\Ex3\hci-ex3\g1-09-ta\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Luca\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AD9F18B-CC4A-4242-A467-A1345B6C56E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B8929B1-1136-4842-AFB9-9A6EBA039E4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="503" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="503" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Background Q" sheetId="3" r:id="rId1"/>
@@ -1414,10 +1414,78 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1434,10 +1502,10 @@
   <a:themeElements>
     <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr val="windowText" lastClr="C6C6C6"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr val="window" lastClr="000000"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -1717,43 +1785,43 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z13"/>
-  <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.54296875" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" customWidth="1"/>
-    <col min="3" max="3" width="11.26953125" customWidth="1"/>
-    <col min="4" max="4" width="5.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" customWidth="1"/>
+    <col min="3" max="3" width="11.28515625" customWidth="1"/>
+    <col min="4" max="4" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="23" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
-    <col min="9" max="9" width="6.7265625" customWidth="1"/>
-    <col min="10" max="10" width="7.81640625" customWidth="1"/>
-    <col min="11" max="11" width="13.54296875" customWidth="1"/>
-    <col min="12" max="12" width="6.26953125" customWidth="1"/>
-    <col min="13" max="13" width="7.1796875" customWidth="1"/>
-    <col min="14" max="14" width="13.54296875" customWidth="1"/>
-    <col min="15" max="15" width="6.26953125" customWidth="1"/>
-    <col min="16" max="16" width="7.54296875" customWidth="1"/>
-    <col min="17" max="17" width="13.453125" customWidth="1"/>
-    <col min="18" max="18" width="12.7265625" customWidth="1"/>
+    <col min="9" max="9" width="6.7109375" customWidth="1"/>
+    <col min="10" max="10" width="7.85546875" customWidth="1"/>
+    <col min="11" max="11" width="13.5703125" customWidth="1"/>
+    <col min="12" max="12" width="6.28515625" customWidth="1"/>
+    <col min="13" max="13" width="7.140625" customWidth="1"/>
+    <col min="14" max="14" width="13.5703125" customWidth="1"/>
+    <col min="15" max="15" width="6.28515625" customWidth="1"/>
+    <col min="16" max="16" width="7.5703125" customWidth="1"/>
+    <col min="17" max="17" width="13.42578125" customWidth="1"/>
+    <col min="18" max="18" width="12.7109375" customWidth="1"/>
     <col min="19" max="19" width="14" customWidth="1"/>
-    <col min="20" max="20" width="8.26953125" customWidth="1"/>
-    <col min="21" max="21" width="15.26953125" customWidth="1"/>
-    <col min="22" max="22" width="13.453125" customWidth="1"/>
-    <col min="23" max="23" width="13.54296875" customWidth="1"/>
-    <col min="24" max="24" width="13.81640625" customWidth="1"/>
-    <col min="25" max="25" width="13.1796875" customWidth="1"/>
-    <col min="26" max="26" width="22.453125" customWidth="1"/>
+    <col min="20" max="20" width="8.28515625" customWidth="1"/>
+    <col min="21" max="21" width="15.28515625" customWidth="1"/>
+    <col min="22" max="22" width="13.42578125" customWidth="1"/>
+    <col min="23" max="23" width="13.5703125" customWidth="1"/>
+    <col min="24" max="24" width="13.85546875" customWidth="1"/>
+    <col min="25" max="25" width="13.140625" customWidth="1"/>
+    <col min="26" max="26" width="22.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:26" s="6" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:26" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C3" s="9" t="s">
         <v>49</v>
       </c>
@@ -1795,7 +1863,7 @@
       <c r="Y3" s="78"/>
       <c r="Z3" s="11"/>
     </row>
-    <row r="4" spans="1:26" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:26" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="31" t="s">
         <v>16</v>
       </c>
@@ -1875,7 +1943,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>17</v>
       </c>
@@ -1955,7 +2023,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
@@ -2035,7 +2103,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
@@ -2115,7 +2183,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -2195,7 +2263,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A9" s="19" t="s">
         <v>21</v>
       </c>
@@ -2275,7 +2343,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="10" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="I10" s="18"/>
       <c r="J10" s="18"/>
       <c r="L10" s="18"/>
@@ -2283,7 +2351,7 @@
       <c r="O10" s="18"/>
       <c r="P10" s="18"/>
     </row>
-    <row r="11" spans="1:26" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A11" s="24"/>
       <c r="B11" s="26" t="s">
         <v>43</v>
@@ -2339,7 +2407,7 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="24"/>
       <c r="B12" s="26" t="s">
         <v>14</v>
@@ -2390,7 +2458,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.2">
       <c r="H13" t="s">
         <v>62</v>
       </c>
@@ -2417,22 +2485,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" style="23" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7265625" customWidth="1"/>
-    <col min="4" max="4" width="15.7265625" customWidth="1"/>
-    <col min="5" max="5" width="11.7265625" customWidth="1"/>
-    <col min="6" max="7" width="10.7265625" customWidth="1"/>
+    <col min="1" max="1" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" style="23" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" customWidth="1"/>
+    <col min="6" max="7" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C3" s="35" t="s">
         <v>4</v>
       </c>
@@ -2441,7 +2509,7 @@
       <c r="F3" s="25"/>
       <c r="G3" s="25"/>
     </row>
-    <row r="4" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="31" t="s">
         <v>16</v>
       </c>
@@ -2464,7 +2532,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>17</v>
       </c>
@@ -2487,7 +2555,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
@@ -2510,7 +2578,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
@@ -2533,7 +2601,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -2556,7 +2624,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
         <v>21</v>
       </c>
@@ -2579,7 +2647,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="24"/>
       <c r="B10" s="24" t="s">
         <v>2</v>
@@ -2605,7 +2673,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="24"/>
       <c r="B11" s="24" t="s">
         <v>3</v>
@@ -2642,29 +2710,29 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K23"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
-    <col min="2" max="2" width="36.1796875" customWidth="1"/>
-    <col min="3" max="3" width="35.1796875" customWidth="1"/>
-    <col min="4" max="4" width="34.453125" customWidth="1"/>
-    <col min="5" max="5" width="25.81640625" customWidth="1"/>
+    <col min="2" max="2" width="36.140625" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" customWidth="1"/>
+    <col min="4" max="4" width="34.42578125" customWidth="1"/>
+    <col min="5" max="5" width="25.85546875" customWidth="1"/>
     <col min="6" max="6" width="29" customWidth="1"/>
-    <col min="7" max="10" width="4.54296875" style="55" customWidth="1"/>
-    <col min="11" max="11" width="6.1796875" style="55" customWidth="1"/>
+    <col min="7" max="10" width="4.5703125" style="55" customWidth="1"/>
+    <col min="11" max="11" width="6.140625" style="55" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="G3" s="58" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:11" s="56" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" s="56" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="60" t="s">
         <v>32</v>
       </c>
@@ -2699,7 +2767,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A5" s="63">
         <v>1</v>
       </c>
@@ -2721,17 +2789,19 @@
       <c r="G5" s="66">
         <v>2</v>
       </c>
-      <c r="H5" s="66"/>
+      <c r="H5" s="66">
+        <v>3</v>
+      </c>
       <c r="I5" s="66"/>
       <c r="J5" s="66">
         <v>2</v>
       </c>
       <c r="K5" s="67">
         <f t="shared" ref="K5:K22" si="0">AVERAGE(G5:J5)</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="37.5" x14ac:dyDescent="0.25">
+        <v>2.3333333333333335</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A6" s="63">
         <v>2</v>
       </c>
@@ -2753,7 +2823,9 @@
       <c r="G6" s="66">
         <v>2</v>
       </c>
-      <c r="H6" s="66"/>
+      <c r="H6" s="66">
+        <v>2</v>
+      </c>
       <c r="I6" s="66"/>
       <c r="J6" s="66">
         <v>2</v>
@@ -2763,7 +2835,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A7" s="63">
         <v>3</v>
       </c>
@@ -2785,7 +2857,9 @@
       <c r="G7" s="66">
         <v>3</v>
       </c>
-      <c r="H7" s="66"/>
+      <c r="H7" s="66">
+        <v>3</v>
+      </c>
       <c r="I7" s="66"/>
       <c r="J7" s="66">
         <v>3</v>
@@ -2795,7 +2869,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A8" s="63">
         <v>4</v>
       </c>
@@ -2817,7 +2891,9 @@
       <c r="G8" s="66">
         <v>1</v>
       </c>
-      <c r="H8" s="66"/>
+      <c r="H8" s="66">
+        <v>1</v>
+      </c>
       <c r="I8" s="66"/>
       <c r="J8" s="66">
         <v>1</v>
@@ -2827,7 +2903,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A9" s="63">
         <v>5</v>
       </c>
@@ -2849,7 +2925,9 @@
       <c r="G9" s="66">
         <v>1</v>
       </c>
-      <c r="H9" s="66"/>
+      <c r="H9" s="66">
+        <v>1</v>
+      </c>
       <c r="I9" s="66">
         <v>2</v>
       </c>
@@ -2858,10 +2936,10 @@
       </c>
       <c r="K9" s="67">
         <f t="shared" si="0"/>
-        <v>1.3333333333333333</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="37.5" x14ac:dyDescent="0.25">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A10" s="63">
         <v>6</v>
       </c>
@@ -2883,7 +2961,9 @@
       <c r="G10" s="66">
         <v>2</v>
       </c>
-      <c r="H10" s="66"/>
+      <c r="H10" s="66">
+        <v>2</v>
+      </c>
       <c r="I10" s="66"/>
       <c r="J10" s="66"/>
       <c r="K10" s="67">
@@ -2891,7 +2971,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A11" s="63">
         <v>7</v>
       </c>
@@ -2913,15 +2993,17 @@
       <c r="G11" s="66">
         <v>2</v>
       </c>
-      <c r="H11" s="66"/>
+      <c r="H11" s="66">
+        <v>3</v>
+      </c>
       <c r="I11" s="66"/>
       <c r="J11" s="66"/>
       <c r="K11" s="67">
         <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A12" s="68" t="s">
         <v>164</v>
       </c>
@@ -2943,7 +3025,9 @@
       <c r="G12" s="66">
         <v>3</v>
       </c>
-      <c r="H12" s="66"/>
+      <c r="H12" s="66">
+        <v>3</v>
+      </c>
       <c r="I12" s="66">
         <v>3</v>
       </c>
@@ -2953,7 +3037,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="50" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A13" s="68" t="s">
         <v>164</v>
       </c>
@@ -2975,17 +3059,19 @@
       <c r="G13" s="66">
         <v>2</v>
       </c>
-      <c r="H13" s="66"/>
+      <c r="H13" s="66">
+        <v>1</v>
+      </c>
       <c r="I13" s="66">
         <v>3</v>
       </c>
       <c r="J13" s="66"/>
       <c r="K13" s="67">
         <f t="shared" si="0"/>
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="50" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A14" s="68" t="s">
         <v>164</v>
       </c>
@@ -3007,7 +3093,9 @@
       <c r="G14" s="66">
         <v>3</v>
       </c>
-      <c r="H14" s="66"/>
+      <c r="H14" s="66">
+        <v>3</v>
+      </c>
       <c r="I14" s="66">
         <v>3</v>
       </c>
@@ -3017,7 +3105,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="50" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A15" s="68" t="s">
         <v>164</v>
       </c>
@@ -3039,17 +3127,19 @@
       <c r="G15" s="66">
         <v>2</v>
       </c>
-      <c r="H15" s="66"/>
+      <c r="H15" s="66">
+        <v>3</v>
+      </c>
       <c r="I15" s="66">
         <v>2</v>
       </c>
       <c r="J15" s="66"/>
       <c r="K15" s="67">
         <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
+        <v>2.3333333333333335</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A16" s="68" t="s">
         <v>164</v>
       </c>
@@ -3071,17 +3161,19 @@
       <c r="G16" s="66">
         <v>1</v>
       </c>
-      <c r="H16" s="66"/>
+      <c r="H16" s="66">
+        <v>2</v>
+      </c>
       <c r="I16" s="66">
         <v>2</v>
       </c>
       <c r="J16" s="66"/>
       <c r="K16" s="67">
         <f t="shared" si="0"/>
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="50" x14ac:dyDescent="0.25">
+        <v>1.6666666666666667</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A17" s="68" t="s">
         <v>164</v>
       </c>
@@ -3103,17 +3195,19 @@
       <c r="G17" s="66">
         <v>1</v>
       </c>
-      <c r="H17" s="66"/>
+      <c r="H17" s="66">
+        <v>2</v>
+      </c>
       <c r="I17" s="66">
         <v>2</v>
       </c>
       <c r="J17" s="66"/>
       <c r="K17" s="67">
         <f t="shared" si="0"/>
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="50" x14ac:dyDescent="0.25">
+        <v>1.6666666666666667</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A18" s="68" t="s">
         <v>164</v>
       </c>
@@ -3135,17 +3229,19 @@
       <c r="G18" s="66">
         <v>1</v>
       </c>
-      <c r="H18" s="66"/>
+      <c r="H18" s="66">
+        <v>1</v>
+      </c>
       <c r="I18" s="66">
         <v>2</v>
       </c>
       <c r="J18" s="66"/>
       <c r="K18" s="67">
         <f t="shared" si="0"/>
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
+        <v>1.3333333333333333</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A19" s="68" t="s">
         <v>164</v>
       </c>
@@ -3167,17 +3263,19 @@
       <c r="G19" s="66">
         <v>2</v>
       </c>
-      <c r="H19" s="66"/>
+      <c r="H19" s="66">
+        <v>3</v>
+      </c>
       <c r="I19" s="66">
         <v>2</v>
       </c>
       <c r="J19" s="66"/>
       <c r="K19" s="67">
         <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="50" x14ac:dyDescent="0.25">
+        <v>2.3333333333333335</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A20" s="68" t="s">
         <v>164</v>
       </c>
@@ -3207,7 +3305,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A21" s="68" t="s">
         <v>164</v>
       </c>
@@ -3237,7 +3335,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A22" s="68" t="s">
         <v>164</v>
       </c>
@@ -3259,12 +3357,15 @@
       <c r="G22" s="55">
         <v>2</v>
       </c>
+      <c r="H22" s="55">
+        <v>2</v>
+      </c>
       <c r="K22" s="67">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" s="68"/>
       <c r="K23" s="67"/>
     </row>
@@ -3277,28 +3378,28 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K14"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
-    <col min="3" max="4" width="35.1796875" customWidth="1"/>
-    <col min="5" max="5" width="26.1796875" customWidth="1"/>
-    <col min="6" max="6" width="29.1796875" customWidth="1"/>
-    <col min="7" max="10" width="4.54296875" style="55" customWidth="1"/>
-    <col min="11" max="11" width="5.81640625" style="55" customWidth="1"/>
+    <col min="3" max="4" width="35.140625" customWidth="1"/>
+    <col min="5" max="5" width="26.140625" customWidth="1"/>
+    <col min="6" max="6" width="29.140625" customWidth="1"/>
+    <col min="7" max="10" width="4.5703125" style="55" customWidth="1"/>
+    <col min="11" max="11" width="5.85546875" style="55" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="G3" s="58" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:11" s="56" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" s="56" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="60" t="s">
         <v>32</v>
       </c>
@@ -3333,7 +3434,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A5" s="63">
         <v>1</v>
       </c>
@@ -3355,7 +3456,9 @@
       <c r="G5" s="66">
         <v>2</v>
       </c>
-      <c r="H5" s="66"/>
+      <c r="H5" s="66">
+        <v>2</v>
+      </c>
       <c r="I5" s="66"/>
       <c r="J5" s="66">
         <v>2</v>
@@ -3365,7 +3468,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A6" s="63">
         <v>2</v>
       </c>
@@ -3387,7 +3490,9 @@
       <c r="G6" s="66">
         <v>2</v>
       </c>
-      <c r="H6" s="66"/>
+      <c r="H6" s="66">
+        <v>2</v>
+      </c>
       <c r="I6" s="66"/>
       <c r="J6" s="66"/>
       <c r="K6" s="67">
@@ -3395,7 +3500,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A7" s="63" t="s">
         <v>164</v>
       </c>
@@ -3417,17 +3522,19 @@
       <c r="G7" s="66">
         <v>2</v>
       </c>
-      <c r="H7" s="66"/>
+      <c r="H7" s="66">
+        <v>3</v>
+      </c>
       <c r="I7" s="66">
         <v>3</v>
       </c>
       <c r="J7" s="66"/>
       <c r="K7" s="67">
         <f t="shared" si="0"/>
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="50" x14ac:dyDescent="0.25">
+        <v>2.6666666666666665</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A8" s="63" t="s">
         <v>164</v>
       </c>
@@ -3449,17 +3556,19 @@
       <c r="G8" s="66">
         <v>2</v>
       </c>
-      <c r="H8" s="66"/>
+      <c r="H8" s="66">
+        <v>2</v>
+      </c>
       <c r="I8" s="66">
         <v>3</v>
       </c>
       <c r="J8" s="66"/>
       <c r="K8" s="67">
         <f t="shared" si="0"/>
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="25" x14ac:dyDescent="0.25">
+        <v>2.3333333333333335</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A9" s="63" t="s">
         <v>164</v>
       </c>
@@ -3481,17 +3590,19 @@
       <c r="G9" s="66">
         <v>2</v>
       </c>
-      <c r="H9" s="66"/>
+      <c r="H9" s="66">
+        <v>1</v>
+      </c>
       <c r="I9" s="66">
         <v>1</v>
       </c>
       <c r="J9" s="66"/>
       <c r="K9" s="67">
         <f t="shared" si="0"/>
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="50" x14ac:dyDescent="0.25">
+        <v>1.3333333333333333</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A10" s="63" t="s">
         <v>164</v>
       </c>
@@ -3523,7 +3634,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="25" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A11" s="63" t="s">
         <v>164</v>
       </c>
@@ -3555,7 +3666,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A12" s="63" t="s">
         <v>164</v>
       </c>
@@ -3587,7 +3698,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="63"/>
       <c r="B13" s="64"/>
       <c r="C13" s="64"/>
@@ -3600,7 +3711,7 @@
       <c r="J13" s="66"/>
       <c r="K13" s="67"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" s="63"/>
       <c r="B14" s="64"/>
       <c r="C14" s="64"/>
@@ -3622,46 +3733,46 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:Q11"/>
-  <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" style="23" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="27.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="32.1796875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="29.1796875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="24.1796875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20.1796875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="24.453125" customWidth="1"/>
-    <col min="16" max="17" width="20.1796875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="22.1796875" customWidth="1"/>
+    <col min="1" max="1" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" style="23" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="32.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="24.42578125" customWidth="1"/>
+    <col min="16" max="17" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="22.140625" customWidth="1"/>
     <col min="19" max="19" width="22" customWidth="1"/>
-    <col min="20" max="20" width="15.7265625" customWidth="1"/>
+    <col min="20" max="20" width="15.7109375" customWidth="1"/>
     <col min="21" max="21" width="14" customWidth="1"/>
-    <col min="22" max="22" width="17.54296875" customWidth="1"/>
+    <col min="22" max="22" width="17.5703125" customWidth="1"/>
     <col min="23" max="23" width="16" customWidth="1"/>
     <col min="24" max="24" width="25" customWidth="1"/>
-    <col min="25" max="25" width="19.81640625" customWidth="1"/>
-    <col min="26" max="26" width="10.1796875" customWidth="1"/>
-    <col min="27" max="27" width="7.81640625" customWidth="1"/>
-    <col min="28" max="28" width="8.7265625" customWidth="1"/>
-    <col min="29" max="29" width="9.54296875" customWidth="1"/>
-    <col min="30" max="30" width="8.7265625" customWidth="1"/>
-    <col min="31" max="31" width="29.453125" customWidth="1"/>
+    <col min="25" max="25" width="19.85546875" customWidth="1"/>
+    <col min="26" max="26" width="10.140625" customWidth="1"/>
+    <col min="27" max="27" width="7.85546875" customWidth="1"/>
+    <col min="28" max="28" width="8.7109375" customWidth="1"/>
+    <col min="29" max="29" width="9.5703125" customWidth="1"/>
+    <col min="30" max="30" width="8.7109375" customWidth="1"/>
+    <col min="31" max="31" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="3" spans="1:17" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:17" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="31" t="s">
         <v>16</v>
       </c>
@@ -3714,7 +3825,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="4" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>17</v>
       </c>
@@ -3767,7 +3878,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
@@ -3820,7 +3931,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>19</v>
       </c>
@@ -3873,7 +3984,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -3926,7 +4037,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:17" s="18" customFormat="1" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" s="18" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>21</v>
       </c>
@@ -3979,7 +4090,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C9" s="18"/>
       <c r="D9" s="18"/>
       <c r="E9" s="18"/>
@@ -3992,7 +4103,7 @@
       <c r="L9" s="18"/>
       <c r="M9" s="18"/>
     </row>
-    <row r="10" spans="1:17" s="18" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="24"/>
       <c r="B10" s="24" t="s">
         <v>43</v>
@@ -4058,7 +4169,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:17" s="18" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:17" s="18" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="24"/>
       <c r="B11" s="24" t="s">
         <v>5</v>

</xml_diff>

<commit_message>
Added Fabian Ratings of findings
</commit_message>
<xml_diff>
--- a/g1-09-ta/data-ta.xlsx
+++ b/g1-09-ta/data-ta.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Luca\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Uni\HCI\hci-ex3\g1-09-ta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B8929B1-1136-4842-AFB9-9A6EBA039E4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67D3275F-4349-43B2-A35A-86024459A47B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="503" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="503" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Background Q" sheetId="3" r:id="rId1"/>
@@ -1414,78 +1414,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1502,10 +1434,10 @@
   <a:themeElements>
     <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="C6C6C6"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="000000"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -1785,7 +1717,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z13"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.5703125" customWidth="1"/>
     <col min="2" max="2" width="12.140625" customWidth="1"/>
@@ -2485,7 +2417,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.140625" style="23" bestFit="1" customWidth="1"/>
@@ -2710,7 +2642,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K23"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
     <col min="2" max="2" width="36.140625" customWidth="1"/>
@@ -2801,7 +2733,7 @@
         <v>2.3333333333333335</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A6" s="63">
         <v>2</v>
       </c>
@@ -2965,10 +2897,12 @@
         <v>2</v>
       </c>
       <c r="I10" s="66"/>
-      <c r="J10" s="66"/>
+      <c r="J10" s="66">
+        <v>3</v>
+      </c>
       <c r="K10" s="67">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>2.3333333333333335</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="51" x14ac:dyDescent="0.2">
@@ -2997,10 +2931,12 @@
         <v>3</v>
       </c>
       <c r="I11" s="66"/>
-      <c r="J11" s="66"/>
+      <c r="J11" s="66">
+        <v>2</v>
+      </c>
       <c r="K11" s="67">
         <f t="shared" si="0"/>
-        <v>2.5</v>
+        <v>2.3333333333333335</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
@@ -3031,7 +2967,9 @@
       <c r="I12" s="66">
         <v>3</v>
       </c>
-      <c r="J12" s="66"/>
+      <c r="J12" s="66">
+        <v>3</v>
+      </c>
       <c r="K12" s="67">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -3065,10 +3003,12 @@
       <c r="I13" s="66">
         <v>3</v>
       </c>
-      <c r="J13" s="66"/>
+      <c r="J13" s="66">
+        <v>3</v>
+      </c>
       <c r="K13" s="67">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="51" x14ac:dyDescent="0.2">
@@ -3099,10 +3039,12 @@
       <c r="I14" s="66">
         <v>3</v>
       </c>
-      <c r="J14" s="66"/>
+      <c r="J14" s="66">
+        <v>4</v>
+      </c>
       <c r="K14" s="67">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="51" x14ac:dyDescent="0.2">
@@ -3133,10 +3075,12 @@
       <c r="I15" s="66">
         <v>2</v>
       </c>
-      <c r="J15" s="66"/>
+      <c r="J15" s="66">
+        <v>3</v>
+      </c>
       <c r="K15" s="67">
         <f t="shared" si="0"/>
-        <v>2.3333333333333335</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
@@ -3167,10 +3111,12 @@
       <c r="I16" s="66">
         <v>2</v>
       </c>
-      <c r="J16" s="66"/>
+      <c r="J16" s="66">
+        <v>1</v>
+      </c>
       <c r="K16" s="67">
         <f t="shared" si="0"/>
-        <v>1.6666666666666667</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="51" x14ac:dyDescent="0.2">
@@ -3201,10 +3147,12 @@
       <c r="I17" s="66">
         <v>2</v>
       </c>
-      <c r="J17" s="66"/>
+      <c r="J17" s="66">
+        <v>3</v>
+      </c>
       <c r="K17" s="67">
         <f t="shared" si="0"/>
-        <v>1.6666666666666667</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="51" x14ac:dyDescent="0.2">
@@ -3235,10 +3183,12 @@
       <c r="I18" s="66">
         <v>2</v>
       </c>
-      <c r="J18" s="66"/>
+      <c r="J18" s="66">
+        <v>0</v>
+      </c>
       <c r="K18" s="67">
         <f t="shared" si="0"/>
-        <v>1.3333333333333333</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
@@ -3269,10 +3219,12 @@
       <c r="I19" s="66">
         <v>2</v>
       </c>
-      <c r="J19" s="66"/>
+      <c r="J19" s="66">
+        <v>4</v>
+      </c>
       <c r="K19" s="67">
         <f t="shared" si="0"/>
-        <v>2.3333333333333335</v>
+        <v>2.75</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
@@ -3300,9 +3252,12 @@
       <c r="H20" s="55">
         <v>3</v>
       </c>
+      <c r="J20" s="55">
+        <v>1</v>
+      </c>
       <c r="K20" s="67">
         <f t="shared" si="0"/>
-        <v>1.5</v>
+        <v>1.3333333333333333</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
@@ -3330,9 +3285,12 @@
       <c r="H21" s="55">
         <v>2</v>
       </c>
+      <c r="J21" s="55">
+        <v>2</v>
+      </c>
       <c r="K21" s="67">
         <f t="shared" si="0"/>
-        <v>2.5</v>
+        <v>2.3333333333333335</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
@@ -3360,9 +3318,12 @@
       <c r="H22" s="55">
         <v>2</v>
       </c>
+      <c r="J22" s="55">
+        <v>3</v>
+      </c>
       <c r="K22" s="67">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>2.3333333333333335</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
@@ -3378,7 +3339,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K14"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
@@ -3494,10 +3455,12 @@
         <v>2</v>
       </c>
       <c r="I6" s="66"/>
-      <c r="J6" s="66"/>
+      <c r="J6" s="66">
+        <v>3</v>
+      </c>
       <c r="K6" s="67">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>2.3333333333333335</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="76.5" x14ac:dyDescent="0.2">
@@ -3528,10 +3491,12 @@
       <c r="I7" s="66">
         <v>3</v>
       </c>
-      <c r="J7" s="66"/>
+      <c r="J7" s="66">
+        <v>4</v>
+      </c>
       <c r="K7" s="67">
         <f t="shared" si="0"/>
-        <v>2.6666666666666665</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="51" x14ac:dyDescent="0.2">
@@ -3562,10 +3527,12 @@
       <c r="I8" s="66">
         <v>3</v>
       </c>
-      <c r="J8" s="66"/>
+      <c r="J8" s="66">
+        <v>2</v>
+      </c>
       <c r="K8" s="67">
         <f t="shared" si="0"/>
-        <v>2.3333333333333335</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
@@ -3596,10 +3563,12 @@
       <c r="I9" s="66">
         <v>1</v>
       </c>
-      <c r="J9" s="66"/>
+      <c r="J9" s="66">
+        <v>1</v>
+      </c>
       <c r="K9" s="67">
         <f t="shared" si="0"/>
-        <v>1.3333333333333333</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
@@ -3628,7 +3597,9 @@
         <v>3</v>
       </c>
       <c r="I10" s="66"/>
-      <c r="J10" s="66"/>
+      <c r="J10" s="66">
+        <v>3</v>
+      </c>
       <c r="K10" s="67">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -3660,10 +3631,12 @@
         <v>2</v>
       </c>
       <c r="I11" s="66"/>
-      <c r="J11" s="66"/>
+      <c r="J11" s="66">
+        <v>4</v>
+      </c>
       <c r="K11" s="67">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>2.6666666666666665</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
@@ -3692,7 +3665,9 @@
         <v>3</v>
       </c>
       <c r="I12" s="66"/>
-      <c r="J12" s="66"/>
+      <c r="J12" s="66">
+        <v>3</v>
+      </c>
       <c r="K12" s="67">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -3733,7 +3708,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:Q11"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.140625" style="23" bestFit="1" customWidth="1"/>

</xml_diff>